<commit_message>
Update Primera FEB 2025-26 boxscore XLSX
Refresh raw boxscore_full_analysis .xlsx files for the Primera FEB 2025-26 Regular_Season. Twenty binary Excel files under informes_data/Primera FEB/2025-26/Regular_Season/raw were modified (boxscore_full_analysis_<id>_LIGAREGULAR...xlsx). Changes appear to be data refreshes or corrections to the regular-season boxscore exports.
</commit_message>
<xml_diff>
--- a/informes_data/Primera FEB/2025-26/Regular_Season/raw/boxscore_full_analysis_2486351_LIGAREGULARÚNICO.xlsx
+++ b/informes_data/Primera FEB/2025-26/Regular_Season/raw/boxscore_full_analysis_2486351_LIGAREGULARÚNICO.xlsx
@@ -614,6 +614,21 @@
           <t>Gen/TO</t>
         </is>
       </c>
+      <c r="AL1" s="1" t="inlineStr"/>
+      <c r="AM1" s="1" t="inlineStr"/>
+      <c r="AN1" s="1" t="inlineStr"/>
+      <c r="AO1" s="1" t="inlineStr"/>
+      <c r="AP1" s="1" t="inlineStr"/>
+      <c r="AQ1" s="1" t="inlineStr"/>
+      <c r="AR1" s="1" t="inlineStr"/>
+      <c r="AS1" s="1" t="inlineStr"/>
+      <c r="AT1" s="1" t="inlineStr"/>
+      <c r="AU1" s="1" t="inlineStr"/>
+      <c r="AV1" s="1" t="inlineStr"/>
+      <c r="AW1" s="1" t="inlineStr"/>
+      <c r="AX1" s="1" t="inlineStr"/>
+      <c r="AY1" s="1" t="inlineStr"/>
+      <c r="AZ1" s="1" t="inlineStr"/>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -773,11 +788,26 @@
           <t>6.38</t>
         </is>
       </c>
+      <c r="AL2" t="inlineStr"/>
+      <c r="AM2" t="inlineStr"/>
+      <c r="AN2" t="inlineStr"/>
+      <c r="AO2" t="inlineStr"/>
+      <c r="AP2" t="inlineStr"/>
+      <c r="AQ2" t="inlineStr"/>
+      <c r="AR2" t="inlineStr"/>
+      <c r="AS2" t="inlineStr"/>
+      <c r="AT2" t="inlineStr"/>
+      <c r="AU2" t="inlineStr"/>
+      <c r="AV2" t="inlineStr"/>
+      <c r="AW2" t="inlineStr"/>
+      <c r="AX2" t="inlineStr"/>
+      <c r="AY2" t="inlineStr"/>
+      <c r="AZ2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>CLOUD.GAL OURENSE BALONCESTO</t>
+          <t>CLUB OURENSE BALONCESTO</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -932,6 +962,75 @@
           <t>13.00</t>
         </is>
       </c>
+      <c r="AL3" t="inlineStr"/>
+      <c r="AM3" t="inlineStr"/>
+      <c r="AN3" t="inlineStr"/>
+      <c r="AO3" t="inlineStr"/>
+      <c r="AP3" t="inlineStr"/>
+      <c r="AQ3" t="inlineStr"/>
+      <c r="AR3" t="inlineStr"/>
+      <c r="AS3" t="inlineStr"/>
+      <c r="AT3" t="inlineStr"/>
+      <c r="AU3" t="inlineStr"/>
+      <c r="AV3" t="inlineStr"/>
+      <c r="AW3" t="inlineStr"/>
+      <c r="AX3" t="inlineStr"/>
+      <c r="AY3" t="inlineStr"/>
+      <c r="AZ3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr"/>
+      <c r="B4" t="inlineStr"/>
+      <c r="C4" t="inlineStr"/>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr"/>
+      <c r="N4" t="inlineStr"/>
+      <c r="O4" t="inlineStr"/>
+      <c r="P4" t="inlineStr"/>
+      <c r="Q4" t="inlineStr"/>
+      <c r="R4" t="inlineStr"/>
+      <c r="S4" t="inlineStr"/>
+      <c r="T4" t="inlineStr"/>
+      <c r="U4" t="inlineStr"/>
+      <c r="V4" t="inlineStr"/>
+      <c r="W4" t="inlineStr"/>
+      <c r="X4" t="inlineStr"/>
+      <c r="Y4" t="inlineStr"/>
+      <c r="Z4" t="inlineStr"/>
+      <c r="AA4" t="inlineStr"/>
+      <c r="AB4" t="inlineStr"/>
+      <c r="AC4" t="inlineStr"/>
+      <c r="AD4" t="inlineStr"/>
+      <c r="AE4" t="inlineStr"/>
+      <c r="AF4" t="inlineStr"/>
+      <c r="AG4" t="inlineStr"/>
+      <c r="AH4" t="inlineStr"/>
+      <c r="AI4" t="inlineStr"/>
+      <c r="AJ4" t="inlineStr"/>
+      <c r="AK4" t="inlineStr"/>
+      <c r="AL4" t="inlineStr"/>
+      <c r="AM4" t="inlineStr"/>
+      <c r="AN4" t="inlineStr"/>
+      <c r="AO4" t="inlineStr"/>
+      <c r="AP4" t="inlineStr"/>
+      <c r="AQ4" t="inlineStr"/>
+      <c r="AR4" t="inlineStr"/>
+      <c r="AS4" t="inlineStr"/>
+      <c r="AT4" t="inlineStr"/>
+      <c r="AU4" t="inlineStr"/>
+      <c r="AV4" t="inlineStr"/>
+      <c r="AW4" t="inlineStr"/>
+      <c r="AX4" t="inlineStr"/>
+      <c r="AY4" t="inlineStr"/>
+      <c r="AZ4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -944,6 +1043,56 @@
           <t>MORALES Gª-ALCAIDE, JUAN P.</t>
         </is>
       </c>
+      <c r="C5" t="inlineStr"/>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr"/>
+      <c r="N5" t="inlineStr"/>
+      <c r="O5" t="inlineStr"/>
+      <c r="P5" t="inlineStr"/>
+      <c r="Q5" t="inlineStr"/>
+      <c r="R5" t="inlineStr"/>
+      <c r="S5" t="inlineStr"/>
+      <c r="T5" t="inlineStr"/>
+      <c r="U5" t="inlineStr"/>
+      <c r="V5" t="inlineStr"/>
+      <c r="W5" t="inlineStr"/>
+      <c r="X5" t="inlineStr"/>
+      <c r="Y5" t="inlineStr"/>
+      <c r="Z5" t="inlineStr"/>
+      <c r="AA5" t="inlineStr"/>
+      <c r="AB5" t="inlineStr"/>
+      <c r="AC5" t="inlineStr"/>
+      <c r="AD5" t="inlineStr"/>
+      <c r="AE5" t="inlineStr"/>
+      <c r="AF5" t="inlineStr"/>
+      <c r="AG5" t="inlineStr"/>
+      <c r="AH5" t="inlineStr"/>
+      <c r="AI5" t="inlineStr"/>
+      <c r="AJ5" t="inlineStr"/>
+      <c r="AK5" t="inlineStr"/>
+      <c r="AL5" t="inlineStr"/>
+      <c r="AM5" t="inlineStr"/>
+      <c r="AN5" t="inlineStr"/>
+      <c r="AO5" t="inlineStr"/>
+      <c r="AP5" t="inlineStr"/>
+      <c r="AQ5" t="inlineStr"/>
+      <c r="AR5" t="inlineStr"/>
+      <c r="AS5" t="inlineStr"/>
+      <c r="AT5" t="inlineStr"/>
+      <c r="AU5" t="inlineStr"/>
+      <c r="AV5" t="inlineStr"/>
+      <c r="AW5" t="inlineStr"/>
+      <c r="AX5" t="inlineStr"/>
+      <c r="AY5" t="inlineStr"/>
+      <c r="AZ5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -956,6 +1105,56 @@
           <t>RODRIGUEZ FERNANDEZ, PABLO</t>
         </is>
       </c>
+      <c r="C6" t="inlineStr"/>
+      <c r="D6" t="inlineStr"/>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="inlineStr"/>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr"/>
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="inlineStr"/>
+      <c r="N6" t="inlineStr"/>
+      <c r="O6" t="inlineStr"/>
+      <c r="P6" t="inlineStr"/>
+      <c r="Q6" t="inlineStr"/>
+      <c r="R6" t="inlineStr"/>
+      <c r="S6" t="inlineStr"/>
+      <c r="T6" t="inlineStr"/>
+      <c r="U6" t="inlineStr"/>
+      <c r="V6" t="inlineStr"/>
+      <c r="W6" t="inlineStr"/>
+      <c r="X6" t="inlineStr"/>
+      <c r="Y6" t="inlineStr"/>
+      <c r="Z6" t="inlineStr"/>
+      <c r="AA6" t="inlineStr"/>
+      <c r="AB6" t="inlineStr"/>
+      <c r="AC6" t="inlineStr"/>
+      <c r="AD6" t="inlineStr"/>
+      <c r="AE6" t="inlineStr"/>
+      <c r="AF6" t="inlineStr"/>
+      <c r="AG6" t="inlineStr"/>
+      <c r="AH6" t="inlineStr"/>
+      <c r="AI6" t="inlineStr"/>
+      <c r="AJ6" t="inlineStr"/>
+      <c r="AK6" t="inlineStr"/>
+      <c r="AL6" t="inlineStr"/>
+      <c r="AM6" t="inlineStr"/>
+      <c r="AN6" t="inlineStr"/>
+      <c r="AO6" t="inlineStr"/>
+      <c r="AP6" t="inlineStr"/>
+      <c r="AQ6" t="inlineStr"/>
+      <c r="AR6" t="inlineStr"/>
+      <c r="AS6" t="inlineStr"/>
+      <c r="AT6" t="inlineStr"/>
+      <c r="AU6" t="inlineStr"/>
+      <c r="AV6" t="inlineStr"/>
+      <c r="AW6" t="inlineStr"/>
+      <c r="AX6" t="inlineStr"/>
+      <c r="AY6" t="inlineStr"/>
+      <c r="AZ6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -968,6 +1167,56 @@
           <t>FERNANDO MARTIN, PABELLON</t>
         </is>
       </c>
+      <c r="C7" t="inlineStr"/>
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr"/>
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr"/>
+      <c r="L7" t="inlineStr"/>
+      <c r="M7" t="inlineStr"/>
+      <c r="N7" t="inlineStr"/>
+      <c r="O7" t="inlineStr"/>
+      <c r="P7" t="inlineStr"/>
+      <c r="Q7" t="inlineStr"/>
+      <c r="R7" t="inlineStr"/>
+      <c r="S7" t="inlineStr"/>
+      <c r="T7" t="inlineStr"/>
+      <c r="U7" t="inlineStr"/>
+      <c r="V7" t="inlineStr"/>
+      <c r="W7" t="inlineStr"/>
+      <c r="X7" t="inlineStr"/>
+      <c r="Y7" t="inlineStr"/>
+      <c r="Z7" t="inlineStr"/>
+      <c r="AA7" t="inlineStr"/>
+      <c r="AB7" t="inlineStr"/>
+      <c r="AC7" t="inlineStr"/>
+      <c r="AD7" t="inlineStr"/>
+      <c r="AE7" t="inlineStr"/>
+      <c r="AF7" t="inlineStr"/>
+      <c r="AG7" t="inlineStr"/>
+      <c r="AH7" t="inlineStr"/>
+      <c r="AI7" t="inlineStr"/>
+      <c r="AJ7" t="inlineStr"/>
+      <c r="AK7" t="inlineStr"/>
+      <c r="AL7" t="inlineStr"/>
+      <c r="AM7" t="inlineStr"/>
+      <c r="AN7" t="inlineStr"/>
+      <c r="AO7" t="inlineStr"/>
+      <c r="AP7" t="inlineStr"/>
+      <c r="AQ7" t="inlineStr"/>
+      <c r="AR7" t="inlineStr"/>
+      <c r="AS7" t="inlineStr"/>
+      <c r="AT7" t="inlineStr"/>
+      <c r="AU7" t="inlineStr"/>
+      <c r="AV7" t="inlineStr"/>
+      <c r="AW7" t="inlineStr"/>
+      <c r="AX7" t="inlineStr"/>
+      <c r="AY7" t="inlineStr"/>
+      <c r="AZ7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -980,6 +1229,164 @@
           <t>GRECIA, S/N, Madrid (Fuenlabrada)</t>
         </is>
       </c>
+      <c r="C8" t="inlineStr"/>
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr"/>
+      <c r="L8" t="inlineStr"/>
+      <c r="M8" t="inlineStr"/>
+      <c r="N8" t="inlineStr"/>
+      <c r="O8" t="inlineStr"/>
+      <c r="P8" t="inlineStr"/>
+      <c r="Q8" t="inlineStr"/>
+      <c r="R8" t="inlineStr"/>
+      <c r="S8" t="inlineStr"/>
+      <c r="T8" t="inlineStr"/>
+      <c r="U8" t="inlineStr"/>
+      <c r="V8" t="inlineStr"/>
+      <c r="W8" t="inlineStr"/>
+      <c r="X8" t="inlineStr"/>
+      <c r="Y8" t="inlineStr"/>
+      <c r="Z8" t="inlineStr"/>
+      <c r="AA8" t="inlineStr"/>
+      <c r="AB8" t="inlineStr"/>
+      <c r="AC8" t="inlineStr"/>
+      <c r="AD8" t="inlineStr"/>
+      <c r="AE8" t="inlineStr"/>
+      <c r="AF8" t="inlineStr"/>
+      <c r="AG8" t="inlineStr"/>
+      <c r="AH8" t="inlineStr"/>
+      <c r="AI8" t="inlineStr"/>
+      <c r="AJ8" t="inlineStr"/>
+      <c r="AK8" t="inlineStr"/>
+      <c r="AL8" t="inlineStr"/>
+      <c r="AM8" t="inlineStr"/>
+      <c r="AN8" t="inlineStr"/>
+      <c r="AO8" t="inlineStr"/>
+      <c r="AP8" t="inlineStr"/>
+      <c r="AQ8" t="inlineStr"/>
+      <c r="AR8" t="inlineStr"/>
+      <c r="AS8" t="inlineStr"/>
+      <c r="AT8" t="inlineStr"/>
+      <c r="AU8" t="inlineStr"/>
+      <c r="AV8" t="inlineStr"/>
+      <c r="AW8" t="inlineStr"/>
+      <c r="AX8" t="inlineStr"/>
+      <c r="AY8" t="inlineStr"/>
+      <c r="AZ8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr"/>
+      <c r="B9" t="inlineStr"/>
+      <c r="C9" t="inlineStr"/>
+      <c r="D9" t="inlineStr"/>
+      <c r="E9" t="inlineStr"/>
+      <c r="F9" t="inlineStr"/>
+      <c r="G9" t="inlineStr"/>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr"/>
+      <c r="L9" t="inlineStr"/>
+      <c r="M9" t="inlineStr"/>
+      <c r="N9" t="inlineStr"/>
+      <c r="O9" t="inlineStr"/>
+      <c r="P9" t="inlineStr"/>
+      <c r="Q9" t="inlineStr"/>
+      <c r="R9" t="inlineStr"/>
+      <c r="S9" t="inlineStr"/>
+      <c r="T9" t="inlineStr"/>
+      <c r="U9" t="inlineStr"/>
+      <c r="V9" t="inlineStr"/>
+      <c r="W9" t="inlineStr"/>
+      <c r="X9" t="inlineStr"/>
+      <c r="Y9" t="inlineStr"/>
+      <c r="Z9" t="inlineStr"/>
+      <c r="AA9" t="inlineStr"/>
+      <c r="AB9" t="inlineStr"/>
+      <c r="AC9" t="inlineStr"/>
+      <c r="AD9" t="inlineStr"/>
+      <c r="AE9" t="inlineStr"/>
+      <c r="AF9" t="inlineStr"/>
+      <c r="AG9" t="inlineStr"/>
+      <c r="AH9" t="inlineStr"/>
+      <c r="AI9" t="inlineStr"/>
+      <c r="AJ9" t="inlineStr"/>
+      <c r="AK9" t="inlineStr"/>
+      <c r="AL9" t="inlineStr"/>
+      <c r="AM9" t="inlineStr"/>
+      <c r="AN9" t="inlineStr"/>
+      <c r="AO9" t="inlineStr"/>
+      <c r="AP9" t="inlineStr"/>
+      <c r="AQ9" t="inlineStr"/>
+      <c r="AR9" t="inlineStr"/>
+      <c r="AS9" t="inlineStr"/>
+      <c r="AT9" t="inlineStr"/>
+      <c r="AU9" t="inlineStr"/>
+      <c r="AV9" t="inlineStr"/>
+      <c r="AW9" t="inlineStr"/>
+      <c r="AX9" t="inlineStr"/>
+      <c r="AY9" t="inlineStr"/>
+      <c r="AZ9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr"/>
+      <c r="B10" t="inlineStr"/>
+      <c r="C10" t="inlineStr"/>
+      <c r="D10" t="inlineStr"/>
+      <c r="E10" t="inlineStr"/>
+      <c r="F10" t="inlineStr"/>
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr"/>
+      <c r="L10" t="inlineStr"/>
+      <c r="M10" t="inlineStr"/>
+      <c r="N10" t="inlineStr"/>
+      <c r="O10" t="inlineStr"/>
+      <c r="P10" t="inlineStr"/>
+      <c r="Q10" t="inlineStr"/>
+      <c r="R10" t="inlineStr"/>
+      <c r="S10" t="inlineStr"/>
+      <c r="T10" t="inlineStr"/>
+      <c r="U10" t="inlineStr"/>
+      <c r="V10" t="inlineStr"/>
+      <c r="W10" t="inlineStr"/>
+      <c r="X10" t="inlineStr"/>
+      <c r="Y10" t="inlineStr"/>
+      <c r="Z10" t="inlineStr"/>
+      <c r="AA10" t="inlineStr"/>
+      <c r="AB10" t="inlineStr"/>
+      <c r="AC10" t="inlineStr"/>
+      <c r="AD10" t="inlineStr"/>
+      <c r="AE10" t="inlineStr"/>
+      <c r="AF10" t="inlineStr"/>
+      <c r="AG10" t="inlineStr"/>
+      <c r="AH10" t="inlineStr"/>
+      <c r="AI10" t="inlineStr"/>
+      <c r="AJ10" t="inlineStr"/>
+      <c r="AK10" t="inlineStr"/>
+      <c r="AL10" t="inlineStr"/>
+      <c r="AM10" t="inlineStr"/>
+      <c r="AN10" t="inlineStr"/>
+      <c r="AO10" t="inlineStr"/>
+      <c r="AP10" t="inlineStr"/>
+      <c r="AQ10" t="inlineStr"/>
+      <c r="AR10" t="inlineStr"/>
+      <c r="AS10" t="inlineStr"/>
+      <c r="AT10" t="inlineStr"/>
+      <c r="AU10" t="inlineStr"/>
+      <c r="AV10" t="inlineStr"/>
+      <c r="AW10" t="inlineStr"/>
+      <c r="AX10" t="inlineStr"/>
+      <c r="AY10" t="inlineStr"/>
+      <c r="AZ10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -987,264 +1394,315 @@
           <t>FLEXICAR FUENLABRADA</t>
         </is>
       </c>
+      <c r="B11" t="inlineStr"/>
+      <c r="C11" t="inlineStr"/>
+      <c r="D11" t="inlineStr"/>
+      <c r="E11" t="inlineStr"/>
+      <c r="F11" t="inlineStr"/>
+      <c r="G11" t="inlineStr"/>
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr"/>
+      <c r="L11" t="inlineStr"/>
+      <c r="M11" t="inlineStr"/>
+      <c r="N11" t="inlineStr"/>
+      <c r="O11" t="inlineStr"/>
+      <c r="P11" t="inlineStr"/>
+      <c r="Q11" t="inlineStr"/>
+      <c r="R11" t="inlineStr"/>
+      <c r="S11" t="inlineStr"/>
+      <c r="T11" t="inlineStr"/>
+      <c r="U11" t="inlineStr"/>
+      <c r="V11" t="inlineStr"/>
+      <c r="W11" t="inlineStr"/>
+      <c r="X11" t="inlineStr"/>
+      <c r="Y11" t="inlineStr"/>
+      <c r="Z11" t="inlineStr"/>
+      <c r="AA11" t="inlineStr"/>
+      <c r="AB11" t="inlineStr"/>
+      <c r="AC11" t="inlineStr"/>
+      <c r="AD11" t="inlineStr"/>
+      <c r="AE11" t="inlineStr"/>
+      <c r="AF11" t="inlineStr"/>
+      <c r="AG11" t="inlineStr"/>
+      <c r="AH11" t="inlineStr"/>
+      <c r="AI11" t="inlineStr"/>
+      <c r="AJ11" t="inlineStr"/>
+      <c r="AK11" t="inlineStr"/>
+      <c r="AL11" t="inlineStr"/>
+      <c r="AM11" t="inlineStr"/>
+      <c r="AN11" t="inlineStr"/>
+      <c r="AO11" t="inlineStr"/>
+      <c r="AP11" t="inlineStr"/>
+      <c r="AQ11" t="inlineStr"/>
+      <c r="AR11" t="inlineStr"/>
+      <c r="AS11" t="inlineStr"/>
+      <c r="AT11" t="inlineStr"/>
+      <c r="AU11" t="inlineStr"/>
+      <c r="AV11" t="inlineStr"/>
+      <c r="AW11" t="inlineStr"/>
+      <c r="AX11" t="inlineStr"/>
+      <c r="AY11" t="inlineStr"/>
+      <c r="AZ11" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="1" t="inlineStr">
+      <c r="A12" t="inlineStr">
         <is>
           <t>JUGADOR</t>
         </is>
       </c>
-      <c r="B12" s="1" t="inlineStr">
+      <c r="B12" t="inlineStr">
         <is>
           <t>PTS</t>
         </is>
       </c>
-      <c r="C12" s="1" t="inlineStr">
+      <c r="C12" t="inlineStr">
         <is>
           <t>2PM</t>
         </is>
       </c>
-      <c r="D12" s="1" t="inlineStr">
+      <c r="D12" t="inlineStr">
         <is>
           <t>2PA</t>
         </is>
       </c>
-      <c r="E12" s="1" t="inlineStr">
+      <c r="E12" t="inlineStr">
         <is>
           <t>3PM</t>
         </is>
       </c>
-      <c r="F12" s="1" t="inlineStr">
+      <c r="F12" t="inlineStr">
         <is>
           <t>3PA</t>
         </is>
       </c>
-      <c r="G12" s="1" t="inlineStr">
+      <c r="G12" t="inlineStr">
         <is>
           <t>FTM</t>
         </is>
       </c>
-      <c r="H12" s="1" t="inlineStr">
+      <c r="H12" t="inlineStr">
         <is>
           <t>FTA</t>
         </is>
       </c>
-      <c r="I12" s="1" t="inlineStr">
+      <c r="I12" t="inlineStr">
         <is>
           <t>AS</t>
         </is>
       </c>
-      <c r="J12" s="1" t="inlineStr">
+      <c r="J12" t="inlineStr">
         <is>
           <t>DRB</t>
         </is>
       </c>
-      <c r="K12" s="1" t="inlineStr">
+      <c r="K12" t="inlineStr">
         <is>
           <t>ORB</t>
         </is>
       </c>
-      <c r="L12" s="1" t="inlineStr">
+      <c r="L12" t="inlineStr">
         <is>
           <t>STL</t>
         </is>
       </c>
-      <c r="M12" s="1" t="inlineStr">
+      <c r="M12" t="inlineStr">
         <is>
           <t>BLK</t>
         </is>
       </c>
-      <c r="N12" s="1" t="inlineStr">
+      <c r="N12" t="inlineStr">
         <is>
           <t>BLK A.</t>
         </is>
       </c>
-      <c r="O12" s="1" t="inlineStr">
+      <c r="O12" t="inlineStr">
         <is>
           <t>TO</t>
         </is>
       </c>
-      <c r="P12" s="1" t="inlineStr">
+      <c r="P12" t="inlineStr">
         <is>
           <t>TOunf</t>
         </is>
       </c>
-      <c r="Q12" s="1" t="inlineStr">
+      <c r="Q12" t="inlineStr">
         <is>
           <t>F</t>
         </is>
       </c>
-      <c r="R12" s="1" t="inlineStr">
+      <c r="R12" t="inlineStr">
         <is>
           <t>F+</t>
         </is>
       </c>
-      <c r="S12" s="1" t="inlineStr">
+      <c r="S12" t="inlineStr">
         <is>
           <t>EFI</t>
         </is>
       </c>
-      <c r="T12" s="1" t="inlineStr">
+      <c r="T12" t="inlineStr">
         <is>
           <t>TOpts</t>
         </is>
       </c>
-      <c r="U12" s="1" t="inlineStr">
+      <c r="U12" t="inlineStr">
         <is>
           <t>2CPts</t>
         </is>
       </c>
-      <c r="V12" s="1" t="inlineStr">
+      <c r="V12" t="inlineStr">
         <is>
           <t>FastBPts</t>
         </is>
       </c>
-      <c r="W12" s="1" t="inlineStr">
+      <c r="W12" t="inlineStr">
         <is>
           <t>FastB Opp</t>
         </is>
       </c>
-      <c r="X12" s="1" t="inlineStr">
+      <c r="X12" t="inlineStr">
         <is>
           <t>Rim FGM</t>
         </is>
       </c>
-      <c r="Y12" s="1" t="inlineStr">
+      <c r="Y12" t="inlineStr">
         <is>
           <t>Rim FGA</t>
         </is>
       </c>
-      <c r="Z12" s="1" t="inlineStr">
+      <c r="Z12" t="inlineStr">
         <is>
           <t>Rim %</t>
         </is>
       </c>
-      <c r="AA12" s="1" t="inlineStr">
+      <c r="AA12" t="inlineStr">
         <is>
           <t>Paint FGM</t>
         </is>
       </c>
-      <c r="AB12" s="1" t="inlineStr">
+      <c r="AB12" t="inlineStr">
         <is>
           <t>Paint FGA</t>
         </is>
       </c>
-      <c r="AC12" s="1" t="inlineStr">
+      <c r="AC12" t="inlineStr">
         <is>
           <t>Paint %</t>
         </is>
       </c>
-      <c r="AD12" s="1" t="inlineStr">
+      <c r="AD12" t="inlineStr">
         <is>
           <t>MR FGM</t>
         </is>
       </c>
-      <c r="AE12" s="1" t="inlineStr">
+      <c r="AE12" t="inlineStr">
         <is>
           <t>MR FGA</t>
         </is>
       </c>
-      <c r="AF12" s="1" t="inlineStr">
+      <c r="AF12" t="inlineStr">
         <is>
           <t>MR %</t>
         </is>
       </c>
-      <c r="AG12" s="1" t="inlineStr">
+      <c r="AG12" t="inlineStr">
         <is>
           <t>Cor3 FGM</t>
         </is>
       </c>
-      <c r="AH12" s="1" t="inlineStr">
+      <c r="AH12" t="inlineStr">
         <is>
           <t>Cor3 FGA</t>
         </is>
       </c>
-      <c r="AI12" s="1" t="inlineStr">
+      <c r="AI12" t="inlineStr">
         <is>
           <t>Cor3 %</t>
         </is>
       </c>
-      <c r="AJ12" s="1" t="inlineStr">
+      <c r="AJ12" t="inlineStr">
         <is>
           <t>ATB3 FGM</t>
         </is>
       </c>
-      <c r="AK12" s="1" t="inlineStr">
+      <c r="AK12" t="inlineStr">
         <is>
           <t>ATB3 FGA</t>
         </is>
       </c>
-      <c r="AL12" s="1" t="inlineStr">
+      <c r="AL12" t="inlineStr">
         <is>
           <t>ATB3 %</t>
         </is>
       </c>
-      <c r="AM12" s="1" t="inlineStr">
+      <c r="AM12" t="inlineStr">
         <is>
           <t>TIME</t>
         </is>
       </c>
-      <c r="AN12" s="1" t="inlineStr">
+      <c r="AN12" t="inlineStr">
         <is>
           <t>PLAYS</t>
         </is>
       </c>
-      <c r="AO12" s="1" t="inlineStr">
+      <c r="AO12" t="inlineStr">
         <is>
           <t>eFG%</t>
         </is>
       </c>
-      <c r="AP12" s="1" t="inlineStr">
+      <c r="AP12" t="inlineStr">
         <is>
           <t>TS%</t>
         </is>
       </c>
-      <c r="AQ12" s="1" t="inlineStr">
+      <c r="AQ12" t="inlineStr">
         <is>
           <t>PTS/PLAY</t>
         </is>
       </c>
-      <c r="AR12" s="1" t="inlineStr">
+      <c r="AR12" t="inlineStr">
         <is>
           <t>TO%</t>
         </is>
       </c>
-      <c r="AS12" s="1" t="inlineStr">
+      <c r="AS12" t="inlineStr">
         <is>
           <t>FTR</t>
         </is>
       </c>
-      <c r="AT12" s="1" t="inlineStr">
+      <c r="AT12" t="inlineStr">
         <is>
           <t>Ass/TO</t>
         </is>
       </c>
-      <c r="AU12" s="1" t="inlineStr">
+      <c r="AU12" t="inlineStr">
         <is>
           <t>Sh/TO</t>
         </is>
       </c>
-      <c r="AV12" s="1" t="inlineStr">
+      <c r="AV12" t="inlineStr">
         <is>
           <t>Gen/TO</t>
         </is>
       </c>
-      <c r="AW12" s="1" t="inlineStr">
+      <c r="AW12" t="inlineStr">
         <is>
           <t>USG%</t>
         </is>
       </c>
-      <c r="AX12" s="1" t="inlineStr">
+      <c r="AX12" t="inlineStr">
         <is>
           <t>OR%</t>
         </is>
       </c>
-      <c r="AY12" s="1" t="inlineStr">
+      <c r="AY12" t="inlineStr">
         <is>
           <t>DR%</t>
         </is>
       </c>
-      <c r="AZ12" s="1" t="inlineStr">
+      <c r="AZ12" t="inlineStr">
         <is>
           <t>pAST%</t>
         </is>
@@ -3970,270 +4428,375 @@
       </c>
       <c r="AZ26" t="inlineStr"/>
     </row>
+    <row r="27">
+      <c r="A27" t="inlineStr"/>
+      <c r="B27" t="inlineStr"/>
+      <c r="C27" t="inlineStr"/>
+      <c r="D27" t="inlineStr"/>
+      <c r="E27" t="inlineStr"/>
+      <c r="F27" t="inlineStr"/>
+      <c r="G27" t="inlineStr"/>
+      <c r="H27" t="inlineStr"/>
+      <c r="I27" t="inlineStr"/>
+      <c r="J27" t="inlineStr"/>
+      <c r="K27" t="inlineStr"/>
+      <c r="L27" t="inlineStr"/>
+      <c r="M27" t="inlineStr"/>
+      <c r="N27" t="inlineStr"/>
+      <c r="O27" t="inlineStr"/>
+      <c r="P27" t="inlineStr"/>
+      <c r="Q27" t="inlineStr"/>
+      <c r="R27" t="inlineStr"/>
+      <c r="S27" t="inlineStr"/>
+      <c r="T27" t="inlineStr"/>
+      <c r="U27" t="inlineStr"/>
+      <c r="V27" t="inlineStr"/>
+      <c r="W27" t="inlineStr"/>
+      <c r="X27" t="inlineStr"/>
+      <c r="Y27" t="inlineStr"/>
+      <c r="Z27" t="inlineStr"/>
+      <c r="AA27" t="inlineStr"/>
+      <c r="AB27" t="inlineStr"/>
+      <c r="AC27" t="inlineStr"/>
+      <c r="AD27" t="inlineStr"/>
+      <c r="AE27" t="inlineStr"/>
+      <c r="AF27" t="inlineStr"/>
+      <c r="AG27" t="inlineStr"/>
+      <c r="AH27" t="inlineStr"/>
+      <c r="AI27" t="inlineStr"/>
+      <c r="AJ27" t="inlineStr"/>
+      <c r="AK27" t="inlineStr"/>
+      <c r="AL27" t="inlineStr"/>
+      <c r="AM27" t="inlineStr"/>
+      <c r="AN27" t="inlineStr"/>
+      <c r="AO27" t="inlineStr"/>
+      <c r="AP27" t="inlineStr"/>
+      <c r="AQ27" t="inlineStr"/>
+      <c r="AR27" t="inlineStr"/>
+      <c r="AS27" t="inlineStr"/>
+      <c r="AT27" t="inlineStr"/>
+      <c r="AU27" t="inlineStr"/>
+      <c r="AV27" t="inlineStr"/>
+      <c r="AW27" t="inlineStr"/>
+      <c r="AX27" t="inlineStr"/>
+      <c r="AY27" t="inlineStr"/>
+      <c r="AZ27" t="inlineStr"/>
+    </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>CLOUD.GAL OURENSE BALONCESTO</t>
-        </is>
-      </c>
+          <t>CLUB OURENSE BALONCESTO</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr"/>
+      <c r="C28" t="inlineStr"/>
+      <c r="D28" t="inlineStr"/>
+      <c r="E28" t="inlineStr"/>
+      <c r="F28" t="inlineStr"/>
+      <c r="G28" t="inlineStr"/>
+      <c r="H28" t="inlineStr"/>
+      <c r="I28" t="inlineStr"/>
+      <c r="J28" t="inlineStr"/>
+      <c r="K28" t="inlineStr"/>
+      <c r="L28" t="inlineStr"/>
+      <c r="M28" t="inlineStr"/>
+      <c r="N28" t="inlineStr"/>
+      <c r="O28" t="inlineStr"/>
+      <c r="P28" t="inlineStr"/>
+      <c r="Q28" t="inlineStr"/>
+      <c r="R28" t="inlineStr"/>
+      <c r="S28" t="inlineStr"/>
+      <c r="T28" t="inlineStr"/>
+      <c r="U28" t="inlineStr"/>
+      <c r="V28" t="inlineStr"/>
+      <c r="W28" t="inlineStr"/>
+      <c r="X28" t="inlineStr"/>
+      <c r="Y28" t="inlineStr"/>
+      <c r="Z28" t="inlineStr"/>
+      <c r="AA28" t="inlineStr"/>
+      <c r="AB28" t="inlineStr"/>
+      <c r="AC28" t="inlineStr"/>
+      <c r="AD28" t="inlineStr"/>
+      <c r="AE28" t="inlineStr"/>
+      <c r="AF28" t="inlineStr"/>
+      <c r="AG28" t="inlineStr"/>
+      <c r="AH28" t="inlineStr"/>
+      <c r="AI28" t="inlineStr"/>
+      <c r="AJ28" t="inlineStr"/>
+      <c r="AK28" t="inlineStr"/>
+      <c r="AL28" t="inlineStr"/>
+      <c r="AM28" t="inlineStr"/>
+      <c r="AN28" t="inlineStr"/>
+      <c r="AO28" t="inlineStr"/>
+      <c r="AP28" t="inlineStr"/>
+      <c r="AQ28" t="inlineStr"/>
+      <c r="AR28" t="inlineStr"/>
+      <c r="AS28" t="inlineStr"/>
+      <c r="AT28" t="inlineStr"/>
+      <c r="AU28" t="inlineStr"/>
+      <c r="AV28" t="inlineStr"/>
+      <c r="AW28" t="inlineStr"/>
+      <c r="AX28" t="inlineStr"/>
+      <c r="AY28" t="inlineStr"/>
+      <c r="AZ28" t="inlineStr"/>
     </row>
     <row r="29">
-      <c r="A29" s="1" t="inlineStr">
+      <c r="A29" t="inlineStr">
         <is>
           <t>JUGADOR</t>
         </is>
       </c>
-      <c r="B29" s="1" t="inlineStr">
+      <c r="B29" t="inlineStr">
         <is>
           <t>PTS</t>
         </is>
       </c>
-      <c r="C29" s="1" t="inlineStr">
+      <c r="C29" t="inlineStr">
         <is>
           <t>2PM</t>
         </is>
       </c>
-      <c r="D29" s="1" t="inlineStr">
+      <c r="D29" t="inlineStr">
         <is>
           <t>2PA</t>
         </is>
       </c>
-      <c r="E29" s="1" t="inlineStr">
+      <c r="E29" t="inlineStr">
         <is>
           <t>3PM</t>
         </is>
       </c>
-      <c r="F29" s="1" t="inlineStr">
+      <c r="F29" t="inlineStr">
         <is>
           <t>3PA</t>
         </is>
       </c>
-      <c r="G29" s="1" t="inlineStr">
+      <c r="G29" t="inlineStr">
         <is>
           <t>FTM</t>
         </is>
       </c>
-      <c r="H29" s="1" t="inlineStr">
+      <c r="H29" t="inlineStr">
         <is>
           <t>FTA</t>
         </is>
       </c>
-      <c r="I29" s="1" t="inlineStr">
+      <c r="I29" t="inlineStr">
         <is>
           <t>AS</t>
         </is>
       </c>
-      <c r="J29" s="1" t="inlineStr">
+      <c r="J29" t="inlineStr">
         <is>
           <t>DRB</t>
         </is>
       </c>
-      <c r="K29" s="1" t="inlineStr">
+      <c r="K29" t="inlineStr">
         <is>
           <t>ORB</t>
         </is>
       </c>
-      <c r="L29" s="1" t="inlineStr">
+      <c r="L29" t="inlineStr">
         <is>
           <t>STL</t>
         </is>
       </c>
-      <c r="M29" s="1" t="inlineStr">
+      <c r="M29" t="inlineStr">
         <is>
           <t>BLK</t>
         </is>
       </c>
-      <c r="N29" s="1" t="inlineStr">
+      <c r="N29" t="inlineStr">
         <is>
           <t>BLK A.</t>
         </is>
       </c>
-      <c r="O29" s="1" t="inlineStr">
+      <c r="O29" t="inlineStr">
         <is>
           <t>TO</t>
         </is>
       </c>
-      <c r="P29" s="1" t="inlineStr">
+      <c r="P29" t="inlineStr">
         <is>
           <t>TOunf</t>
         </is>
       </c>
-      <c r="Q29" s="1" t="inlineStr">
+      <c r="Q29" t="inlineStr">
         <is>
           <t>F</t>
         </is>
       </c>
-      <c r="R29" s="1" t="inlineStr">
+      <c r="R29" t="inlineStr">
         <is>
           <t>F+</t>
         </is>
       </c>
-      <c r="S29" s="1" t="inlineStr">
+      <c r="S29" t="inlineStr">
         <is>
           <t>EFI</t>
         </is>
       </c>
-      <c r="T29" s="1" t="inlineStr">
+      <c r="T29" t="inlineStr">
         <is>
           <t>TOpts</t>
         </is>
       </c>
-      <c r="U29" s="1" t="inlineStr">
+      <c r="U29" t="inlineStr">
         <is>
           <t>2CPts</t>
         </is>
       </c>
-      <c r="V29" s="1" t="inlineStr">
+      <c r="V29" t="inlineStr">
         <is>
           <t>FastBPts</t>
         </is>
       </c>
-      <c r="W29" s="1" t="inlineStr">
+      <c r="W29" t="inlineStr">
         <is>
           <t>FastB Opp</t>
         </is>
       </c>
-      <c r="X29" s="1" t="inlineStr">
+      <c r="X29" t="inlineStr">
         <is>
           <t>Rim FGM</t>
         </is>
       </c>
-      <c r="Y29" s="1" t="inlineStr">
+      <c r="Y29" t="inlineStr">
         <is>
           <t>Rim FGA</t>
         </is>
       </c>
-      <c r="Z29" s="1" t="inlineStr">
+      <c r="Z29" t="inlineStr">
         <is>
           <t>Rim %</t>
         </is>
       </c>
-      <c r="AA29" s="1" t="inlineStr">
+      <c r="AA29" t="inlineStr">
         <is>
           <t>Paint FGM</t>
         </is>
       </c>
-      <c r="AB29" s="1" t="inlineStr">
+      <c r="AB29" t="inlineStr">
         <is>
           <t>Paint FGA</t>
         </is>
       </c>
-      <c r="AC29" s="1" t="inlineStr">
+      <c r="AC29" t="inlineStr">
         <is>
           <t>Paint %</t>
         </is>
       </c>
-      <c r="AD29" s="1" t="inlineStr">
+      <c r="AD29" t="inlineStr">
         <is>
           <t>MR FGM</t>
         </is>
       </c>
-      <c r="AE29" s="1" t="inlineStr">
+      <c r="AE29" t="inlineStr">
         <is>
           <t>MR FGA</t>
         </is>
       </c>
-      <c r="AF29" s="1" t="inlineStr">
+      <c r="AF29" t="inlineStr">
         <is>
           <t>MR %</t>
         </is>
       </c>
-      <c r="AG29" s="1" t="inlineStr">
+      <c r="AG29" t="inlineStr">
         <is>
           <t>Cor3 FGM</t>
         </is>
       </c>
-      <c r="AH29" s="1" t="inlineStr">
+      <c r="AH29" t="inlineStr">
         <is>
           <t>Cor3 FGA</t>
         </is>
       </c>
-      <c r="AI29" s="1" t="inlineStr">
+      <c r="AI29" t="inlineStr">
         <is>
           <t>Cor3 %</t>
         </is>
       </c>
-      <c r="AJ29" s="1" t="inlineStr">
+      <c r="AJ29" t="inlineStr">
         <is>
           <t>ATB3 FGM</t>
         </is>
       </c>
-      <c r="AK29" s="1" t="inlineStr">
+      <c r="AK29" t="inlineStr">
         <is>
           <t>ATB3 FGA</t>
         </is>
       </c>
-      <c r="AL29" s="1" t="inlineStr">
+      <c r="AL29" t="inlineStr">
         <is>
           <t>ATB3 %</t>
         </is>
       </c>
-      <c r="AM29" s="1" t="inlineStr">
+      <c r="AM29" t="inlineStr">
         <is>
           <t>TIME</t>
         </is>
       </c>
-      <c r="AN29" s="1" t="inlineStr">
+      <c r="AN29" t="inlineStr">
         <is>
           <t>PLAYS</t>
         </is>
       </c>
-      <c r="AO29" s="1" t="inlineStr">
+      <c r="AO29" t="inlineStr">
         <is>
           <t>eFG%</t>
         </is>
       </c>
-      <c r="AP29" s="1" t="inlineStr">
+      <c r="AP29" t="inlineStr">
         <is>
           <t>TS%</t>
         </is>
       </c>
-      <c r="AQ29" s="1" t="inlineStr">
+      <c r="AQ29" t="inlineStr">
         <is>
           <t>PTS/PLAY</t>
         </is>
       </c>
-      <c r="AR29" s="1" t="inlineStr">
+      <c r="AR29" t="inlineStr">
         <is>
           <t>TO%</t>
         </is>
       </c>
-      <c r="AS29" s="1" t="inlineStr">
+      <c r="AS29" t="inlineStr">
         <is>
           <t>FTR</t>
         </is>
       </c>
-      <c r="AT29" s="1" t="inlineStr">
+      <c r="AT29" t="inlineStr">
         <is>
           <t>Ass/TO</t>
         </is>
       </c>
-      <c r="AU29" s="1" t="inlineStr">
+      <c r="AU29" t="inlineStr">
         <is>
           <t>Sh/TO</t>
         </is>
       </c>
-      <c r="AV29" s="1" t="inlineStr">
+      <c r="AV29" t="inlineStr">
         <is>
           <t>Gen/TO</t>
         </is>
       </c>
-      <c r="AW29" s="1" t="inlineStr">
+      <c r="AW29" t="inlineStr">
         <is>
           <t>USG%</t>
         </is>
       </c>
-      <c r="AX29" s="1" t="inlineStr">
+      <c r="AX29" t="inlineStr">
         <is>
           <t>OR%</t>
         </is>
       </c>
-      <c r="AY29" s="1" t="inlineStr">
+      <c r="AY29" t="inlineStr">
         <is>
           <t>DR%</t>
         </is>
       </c>
-      <c r="AZ29" s="1" t="inlineStr">
+      <c r="AZ29" t="inlineStr">
         <is>
           <t>pAST%</t>
         </is>
@@ -6567,24 +7130,179 @@
       </c>
       <c r="AZ41" t="inlineStr"/>
     </row>
+    <row r="42">
+      <c r="A42" t="inlineStr"/>
+      <c r="B42" t="inlineStr"/>
+      <c r="C42" t="inlineStr"/>
+      <c r="D42" t="inlineStr"/>
+      <c r="E42" t="inlineStr"/>
+      <c r="F42" t="inlineStr"/>
+      <c r="G42" t="inlineStr"/>
+      <c r="H42" t="inlineStr"/>
+      <c r="I42" t="inlineStr"/>
+      <c r="J42" t="inlineStr"/>
+      <c r="K42" t="inlineStr"/>
+      <c r="L42" t="inlineStr"/>
+      <c r="M42" t="inlineStr"/>
+      <c r="N42" t="inlineStr"/>
+      <c r="O42" t="inlineStr"/>
+      <c r="P42" t="inlineStr"/>
+      <c r="Q42" t="inlineStr"/>
+      <c r="R42" t="inlineStr"/>
+      <c r="S42" t="inlineStr"/>
+      <c r="T42" t="inlineStr"/>
+      <c r="U42" t="inlineStr"/>
+      <c r="V42" t="inlineStr"/>
+      <c r="W42" t="inlineStr"/>
+      <c r="X42" t="inlineStr"/>
+      <c r="Y42" t="inlineStr"/>
+      <c r="Z42" t="inlineStr"/>
+      <c r="AA42" t="inlineStr"/>
+      <c r="AB42" t="inlineStr"/>
+      <c r="AC42" t="inlineStr"/>
+      <c r="AD42" t="inlineStr"/>
+      <c r="AE42" t="inlineStr"/>
+      <c r="AF42" t="inlineStr"/>
+      <c r="AG42" t="inlineStr"/>
+      <c r="AH42" t="inlineStr"/>
+      <c r="AI42" t="inlineStr"/>
+      <c r="AJ42" t="inlineStr"/>
+      <c r="AK42" t="inlineStr"/>
+      <c r="AL42" t="inlineStr"/>
+      <c r="AM42" t="inlineStr"/>
+      <c r="AN42" t="inlineStr"/>
+      <c r="AO42" t="inlineStr"/>
+      <c r="AP42" t="inlineStr"/>
+      <c r="AQ42" t="inlineStr"/>
+      <c r="AR42" t="inlineStr"/>
+      <c r="AS42" t="inlineStr"/>
+      <c r="AT42" t="inlineStr"/>
+      <c r="AU42" t="inlineStr"/>
+      <c r="AV42" t="inlineStr"/>
+      <c r="AW42" t="inlineStr"/>
+      <c r="AX42" t="inlineStr"/>
+      <c r="AY42" t="inlineStr"/>
+      <c r="AZ42" t="inlineStr"/>
+    </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
           <t>--- Glossary of Terms ---</t>
         </is>
       </c>
+      <c r="B43" t="inlineStr"/>
+      <c r="C43" t="inlineStr"/>
+      <c r="D43" t="inlineStr"/>
+      <c r="E43" t="inlineStr"/>
+      <c r="F43" t="inlineStr"/>
+      <c r="G43" t="inlineStr"/>
+      <c r="H43" t="inlineStr"/>
+      <c r="I43" t="inlineStr"/>
+      <c r="J43" t="inlineStr"/>
+      <c r="K43" t="inlineStr"/>
+      <c r="L43" t="inlineStr"/>
+      <c r="M43" t="inlineStr"/>
+      <c r="N43" t="inlineStr"/>
+      <c r="O43" t="inlineStr"/>
+      <c r="P43" t="inlineStr"/>
+      <c r="Q43" t="inlineStr"/>
+      <c r="R43" t="inlineStr"/>
+      <c r="S43" t="inlineStr"/>
+      <c r="T43" t="inlineStr"/>
+      <c r="U43" t="inlineStr"/>
+      <c r="V43" t="inlineStr"/>
+      <c r="W43" t="inlineStr"/>
+      <c r="X43" t="inlineStr"/>
+      <c r="Y43" t="inlineStr"/>
+      <c r="Z43" t="inlineStr"/>
+      <c r="AA43" t="inlineStr"/>
+      <c r="AB43" t="inlineStr"/>
+      <c r="AC43" t="inlineStr"/>
+      <c r="AD43" t="inlineStr"/>
+      <c r="AE43" t="inlineStr"/>
+      <c r="AF43" t="inlineStr"/>
+      <c r="AG43" t="inlineStr"/>
+      <c r="AH43" t="inlineStr"/>
+      <c r="AI43" t="inlineStr"/>
+      <c r="AJ43" t="inlineStr"/>
+      <c r="AK43" t="inlineStr"/>
+      <c r="AL43" t="inlineStr"/>
+      <c r="AM43" t="inlineStr"/>
+      <c r="AN43" t="inlineStr"/>
+      <c r="AO43" t="inlineStr"/>
+      <c r="AP43" t="inlineStr"/>
+      <c r="AQ43" t="inlineStr"/>
+      <c r="AR43" t="inlineStr"/>
+      <c r="AS43" t="inlineStr"/>
+      <c r="AT43" t="inlineStr"/>
+      <c r="AU43" t="inlineStr"/>
+      <c r="AV43" t="inlineStr"/>
+      <c r="AW43" t="inlineStr"/>
+      <c r="AX43" t="inlineStr"/>
+      <c r="AY43" t="inlineStr"/>
+      <c r="AZ43" t="inlineStr"/>
     </row>
     <row r="44">
-      <c r="A44" s="1" t="inlineStr">
+      <c r="A44" t="inlineStr">
         <is>
           <t>Term</t>
         </is>
       </c>
-      <c r="B44" s="1" t="inlineStr">
+      <c r="B44" t="inlineStr">
         <is>
           <t>Explanation</t>
         </is>
       </c>
+      <c r="C44" t="inlineStr"/>
+      <c r="D44" t="inlineStr"/>
+      <c r="E44" t="inlineStr"/>
+      <c r="F44" t="inlineStr"/>
+      <c r="G44" t="inlineStr"/>
+      <c r="H44" t="inlineStr"/>
+      <c r="I44" t="inlineStr"/>
+      <c r="J44" t="inlineStr"/>
+      <c r="K44" t="inlineStr"/>
+      <c r="L44" t="inlineStr"/>
+      <c r="M44" t="inlineStr"/>
+      <c r="N44" t="inlineStr"/>
+      <c r="O44" t="inlineStr"/>
+      <c r="P44" t="inlineStr"/>
+      <c r="Q44" t="inlineStr"/>
+      <c r="R44" t="inlineStr"/>
+      <c r="S44" t="inlineStr"/>
+      <c r="T44" t="inlineStr"/>
+      <c r="U44" t="inlineStr"/>
+      <c r="V44" t="inlineStr"/>
+      <c r="W44" t="inlineStr"/>
+      <c r="X44" t="inlineStr"/>
+      <c r="Y44" t="inlineStr"/>
+      <c r="Z44" t="inlineStr"/>
+      <c r="AA44" t="inlineStr"/>
+      <c r="AB44" t="inlineStr"/>
+      <c r="AC44" t="inlineStr"/>
+      <c r="AD44" t="inlineStr"/>
+      <c r="AE44" t="inlineStr"/>
+      <c r="AF44" t="inlineStr"/>
+      <c r="AG44" t="inlineStr"/>
+      <c r="AH44" t="inlineStr"/>
+      <c r="AI44" t="inlineStr"/>
+      <c r="AJ44" t="inlineStr"/>
+      <c r="AK44" t="inlineStr"/>
+      <c r="AL44" t="inlineStr"/>
+      <c r="AM44" t="inlineStr"/>
+      <c r="AN44" t="inlineStr"/>
+      <c r="AO44" t="inlineStr"/>
+      <c r="AP44" t="inlineStr"/>
+      <c r="AQ44" t="inlineStr"/>
+      <c r="AR44" t="inlineStr"/>
+      <c r="AS44" t="inlineStr"/>
+      <c r="AT44" t="inlineStr"/>
+      <c r="AU44" t="inlineStr"/>
+      <c r="AV44" t="inlineStr"/>
+      <c r="AW44" t="inlineStr"/>
+      <c r="AX44" t="inlineStr"/>
+      <c r="AY44" t="inlineStr"/>
+      <c r="AZ44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -6597,6 +7315,56 @@
           <t>Efficiency Rating (Official FEB Formula): (PTS + REB + AST + STL + BLK + F+) - (FGA-FGM + FTA-FTM + TO + BLK A. + F)</t>
         </is>
       </c>
+      <c r="C45" t="inlineStr"/>
+      <c r="D45" t="inlineStr"/>
+      <c r="E45" t="inlineStr"/>
+      <c r="F45" t="inlineStr"/>
+      <c r="G45" t="inlineStr"/>
+      <c r="H45" t="inlineStr"/>
+      <c r="I45" t="inlineStr"/>
+      <c r="J45" t="inlineStr"/>
+      <c r="K45" t="inlineStr"/>
+      <c r="L45" t="inlineStr"/>
+      <c r="M45" t="inlineStr"/>
+      <c r="N45" t="inlineStr"/>
+      <c r="O45" t="inlineStr"/>
+      <c r="P45" t="inlineStr"/>
+      <c r="Q45" t="inlineStr"/>
+      <c r="R45" t="inlineStr"/>
+      <c r="S45" t="inlineStr"/>
+      <c r="T45" t="inlineStr"/>
+      <c r="U45" t="inlineStr"/>
+      <c r="V45" t="inlineStr"/>
+      <c r="W45" t="inlineStr"/>
+      <c r="X45" t="inlineStr"/>
+      <c r="Y45" t="inlineStr"/>
+      <c r="Z45" t="inlineStr"/>
+      <c r="AA45" t="inlineStr"/>
+      <c r="AB45" t="inlineStr"/>
+      <c r="AC45" t="inlineStr"/>
+      <c r="AD45" t="inlineStr"/>
+      <c r="AE45" t="inlineStr"/>
+      <c r="AF45" t="inlineStr"/>
+      <c r="AG45" t="inlineStr"/>
+      <c r="AH45" t="inlineStr"/>
+      <c r="AI45" t="inlineStr"/>
+      <c r="AJ45" t="inlineStr"/>
+      <c r="AK45" t="inlineStr"/>
+      <c r="AL45" t="inlineStr"/>
+      <c r="AM45" t="inlineStr"/>
+      <c r="AN45" t="inlineStr"/>
+      <c r="AO45" t="inlineStr"/>
+      <c r="AP45" t="inlineStr"/>
+      <c r="AQ45" t="inlineStr"/>
+      <c r="AR45" t="inlineStr"/>
+      <c r="AS45" t="inlineStr"/>
+      <c r="AT45" t="inlineStr"/>
+      <c r="AU45" t="inlineStr"/>
+      <c r="AV45" t="inlineStr"/>
+      <c r="AW45" t="inlineStr"/>
+      <c r="AX45" t="inlineStr"/>
+      <c r="AY45" t="inlineStr"/>
+      <c r="AZ45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -6609,6 +7377,56 @@
           <t>Blocks Against: A player's shot attempt was blocked by an opponent.</t>
         </is>
       </c>
+      <c r="C46" t="inlineStr"/>
+      <c r="D46" t="inlineStr"/>
+      <c r="E46" t="inlineStr"/>
+      <c r="F46" t="inlineStr"/>
+      <c r="G46" t="inlineStr"/>
+      <c r="H46" t="inlineStr"/>
+      <c r="I46" t="inlineStr"/>
+      <c r="J46" t="inlineStr"/>
+      <c r="K46" t="inlineStr"/>
+      <c r="L46" t="inlineStr"/>
+      <c r="M46" t="inlineStr"/>
+      <c r="N46" t="inlineStr"/>
+      <c r="O46" t="inlineStr"/>
+      <c r="P46" t="inlineStr"/>
+      <c r="Q46" t="inlineStr"/>
+      <c r="R46" t="inlineStr"/>
+      <c r="S46" t="inlineStr"/>
+      <c r="T46" t="inlineStr"/>
+      <c r="U46" t="inlineStr"/>
+      <c r="V46" t="inlineStr"/>
+      <c r="W46" t="inlineStr"/>
+      <c r="X46" t="inlineStr"/>
+      <c r="Y46" t="inlineStr"/>
+      <c r="Z46" t="inlineStr"/>
+      <c r="AA46" t="inlineStr"/>
+      <c r="AB46" t="inlineStr"/>
+      <c r="AC46" t="inlineStr"/>
+      <c r="AD46" t="inlineStr"/>
+      <c r="AE46" t="inlineStr"/>
+      <c r="AF46" t="inlineStr"/>
+      <c r="AG46" t="inlineStr"/>
+      <c r="AH46" t="inlineStr"/>
+      <c r="AI46" t="inlineStr"/>
+      <c r="AJ46" t="inlineStr"/>
+      <c r="AK46" t="inlineStr"/>
+      <c r="AL46" t="inlineStr"/>
+      <c r="AM46" t="inlineStr"/>
+      <c r="AN46" t="inlineStr"/>
+      <c r="AO46" t="inlineStr"/>
+      <c r="AP46" t="inlineStr"/>
+      <c r="AQ46" t="inlineStr"/>
+      <c r="AR46" t="inlineStr"/>
+      <c r="AS46" t="inlineStr"/>
+      <c r="AT46" t="inlineStr"/>
+      <c r="AU46" t="inlineStr"/>
+      <c r="AV46" t="inlineStr"/>
+      <c r="AW46" t="inlineStr"/>
+      <c r="AX46" t="inlineStr"/>
+      <c r="AY46" t="inlineStr"/>
+      <c r="AZ46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -6621,6 +7439,56 @@
           <t>Fouls Received: The number of times a player was fouled by an opponent.</t>
         </is>
       </c>
+      <c r="C47" t="inlineStr"/>
+      <c r="D47" t="inlineStr"/>
+      <c r="E47" t="inlineStr"/>
+      <c r="F47" t="inlineStr"/>
+      <c r="G47" t="inlineStr"/>
+      <c r="H47" t="inlineStr"/>
+      <c r="I47" t="inlineStr"/>
+      <c r="J47" t="inlineStr"/>
+      <c r="K47" t="inlineStr"/>
+      <c r="L47" t="inlineStr"/>
+      <c r="M47" t="inlineStr"/>
+      <c r="N47" t="inlineStr"/>
+      <c r="O47" t="inlineStr"/>
+      <c r="P47" t="inlineStr"/>
+      <c r="Q47" t="inlineStr"/>
+      <c r="R47" t="inlineStr"/>
+      <c r="S47" t="inlineStr"/>
+      <c r="T47" t="inlineStr"/>
+      <c r="U47" t="inlineStr"/>
+      <c r="V47" t="inlineStr"/>
+      <c r="W47" t="inlineStr"/>
+      <c r="X47" t="inlineStr"/>
+      <c r="Y47" t="inlineStr"/>
+      <c r="Z47" t="inlineStr"/>
+      <c r="AA47" t="inlineStr"/>
+      <c r="AB47" t="inlineStr"/>
+      <c r="AC47" t="inlineStr"/>
+      <c r="AD47" t="inlineStr"/>
+      <c r="AE47" t="inlineStr"/>
+      <c r="AF47" t="inlineStr"/>
+      <c r="AG47" t="inlineStr"/>
+      <c r="AH47" t="inlineStr"/>
+      <c r="AI47" t="inlineStr"/>
+      <c r="AJ47" t="inlineStr"/>
+      <c r="AK47" t="inlineStr"/>
+      <c r="AL47" t="inlineStr"/>
+      <c r="AM47" t="inlineStr"/>
+      <c r="AN47" t="inlineStr"/>
+      <c r="AO47" t="inlineStr"/>
+      <c r="AP47" t="inlineStr"/>
+      <c r="AQ47" t="inlineStr"/>
+      <c r="AR47" t="inlineStr"/>
+      <c r="AS47" t="inlineStr"/>
+      <c r="AT47" t="inlineStr"/>
+      <c r="AU47" t="inlineStr"/>
+      <c r="AV47" t="inlineStr"/>
+      <c r="AW47" t="inlineStr"/>
+      <c r="AX47" t="inlineStr"/>
+      <c r="AY47" t="inlineStr"/>
+      <c r="AZ47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -6633,6 +7501,56 @@
           <t>Unforced Turnovers: Turnovers not resulting from a direct steal (e.g., bad pass, out of bounds).</t>
         </is>
       </c>
+      <c r="C48" t="inlineStr"/>
+      <c r="D48" t="inlineStr"/>
+      <c r="E48" t="inlineStr"/>
+      <c r="F48" t="inlineStr"/>
+      <c r="G48" t="inlineStr"/>
+      <c r="H48" t="inlineStr"/>
+      <c r="I48" t="inlineStr"/>
+      <c r="J48" t="inlineStr"/>
+      <c r="K48" t="inlineStr"/>
+      <c r="L48" t="inlineStr"/>
+      <c r="M48" t="inlineStr"/>
+      <c r="N48" t="inlineStr"/>
+      <c r="O48" t="inlineStr"/>
+      <c r="P48" t="inlineStr"/>
+      <c r="Q48" t="inlineStr"/>
+      <c r="R48" t="inlineStr"/>
+      <c r="S48" t="inlineStr"/>
+      <c r="T48" t="inlineStr"/>
+      <c r="U48" t="inlineStr"/>
+      <c r="V48" t="inlineStr"/>
+      <c r="W48" t="inlineStr"/>
+      <c r="X48" t="inlineStr"/>
+      <c r="Y48" t="inlineStr"/>
+      <c r="Z48" t="inlineStr"/>
+      <c r="AA48" t="inlineStr"/>
+      <c r="AB48" t="inlineStr"/>
+      <c r="AC48" t="inlineStr"/>
+      <c r="AD48" t="inlineStr"/>
+      <c r="AE48" t="inlineStr"/>
+      <c r="AF48" t="inlineStr"/>
+      <c r="AG48" t="inlineStr"/>
+      <c r="AH48" t="inlineStr"/>
+      <c r="AI48" t="inlineStr"/>
+      <c r="AJ48" t="inlineStr"/>
+      <c r="AK48" t="inlineStr"/>
+      <c r="AL48" t="inlineStr"/>
+      <c r="AM48" t="inlineStr"/>
+      <c r="AN48" t="inlineStr"/>
+      <c r="AO48" t="inlineStr"/>
+      <c r="AP48" t="inlineStr"/>
+      <c r="AQ48" t="inlineStr"/>
+      <c r="AR48" t="inlineStr"/>
+      <c r="AS48" t="inlineStr"/>
+      <c r="AT48" t="inlineStr"/>
+      <c r="AU48" t="inlineStr"/>
+      <c r="AV48" t="inlineStr"/>
+      <c r="AW48" t="inlineStr"/>
+      <c r="AX48" t="inlineStr"/>
+      <c r="AY48" t="inlineStr"/>
+      <c r="AZ48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -6645,6 +7563,56 @@
           <t>2nd Chance Points: Points scored within 8 seconds immediately following an offensive rebound.</t>
         </is>
       </c>
+      <c r="C49" t="inlineStr"/>
+      <c r="D49" t="inlineStr"/>
+      <c r="E49" t="inlineStr"/>
+      <c r="F49" t="inlineStr"/>
+      <c r="G49" t="inlineStr"/>
+      <c r="H49" t="inlineStr"/>
+      <c r="I49" t="inlineStr"/>
+      <c r="J49" t="inlineStr"/>
+      <c r="K49" t="inlineStr"/>
+      <c r="L49" t="inlineStr"/>
+      <c r="M49" t="inlineStr"/>
+      <c r="N49" t="inlineStr"/>
+      <c r="O49" t="inlineStr"/>
+      <c r="P49" t="inlineStr"/>
+      <c r="Q49" t="inlineStr"/>
+      <c r="R49" t="inlineStr"/>
+      <c r="S49" t="inlineStr"/>
+      <c r="T49" t="inlineStr"/>
+      <c r="U49" t="inlineStr"/>
+      <c r="V49" t="inlineStr"/>
+      <c r="W49" t="inlineStr"/>
+      <c r="X49" t="inlineStr"/>
+      <c r="Y49" t="inlineStr"/>
+      <c r="Z49" t="inlineStr"/>
+      <c r="AA49" t="inlineStr"/>
+      <c r="AB49" t="inlineStr"/>
+      <c r="AC49" t="inlineStr"/>
+      <c r="AD49" t="inlineStr"/>
+      <c r="AE49" t="inlineStr"/>
+      <c r="AF49" t="inlineStr"/>
+      <c r="AG49" t="inlineStr"/>
+      <c r="AH49" t="inlineStr"/>
+      <c r="AI49" t="inlineStr"/>
+      <c r="AJ49" t="inlineStr"/>
+      <c r="AK49" t="inlineStr"/>
+      <c r="AL49" t="inlineStr"/>
+      <c r="AM49" t="inlineStr"/>
+      <c r="AN49" t="inlineStr"/>
+      <c r="AO49" t="inlineStr"/>
+      <c r="AP49" t="inlineStr"/>
+      <c r="AQ49" t="inlineStr"/>
+      <c r="AR49" t="inlineStr"/>
+      <c r="AS49" t="inlineStr"/>
+      <c r="AT49" t="inlineStr"/>
+      <c r="AU49" t="inlineStr"/>
+      <c r="AV49" t="inlineStr"/>
+      <c r="AW49" t="inlineStr"/>
+      <c r="AX49" t="inlineStr"/>
+      <c r="AY49" t="inlineStr"/>
+      <c r="AZ49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -6657,6 +7625,56 @@
           <t>Points off Turnovers: Points scored on any possession that was initiated by an opponent's turnover (possession-based).</t>
         </is>
       </c>
+      <c r="C50" t="inlineStr"/>
+      <c r="D50" t="inlineStr"/>
+      <c r="E50" t="inlineStr"/>
+      <c r="F50" t="inlineStr"/>
+      <c r="G50" t="inlineStr"/>
+      <c r="H50" t="inlineStr"/>
+      <c r="I50" t="inlineStr"/>
+      <c r="J50" t="inlineStr"/>
+      <c r="K50" t="inlineStr"/>
+      <c r="L50" t="inlineStr"/>
+      <c r="M50" t="inlineStr"/>
+      <c r="N50" t="inlineStr"/>
+      <c r="O50" t="inlineStr"/>
+      <c r="P50" t="inlineStr"/>
+      <c r="Q50" t="inlineStr"/>
+      <c r="R50" t="inlineStr"/>
+      <c r="S50" t="inlineStr"/>
+      <c r="T50" t="inlineStr"/>
+      <c r="U50" t="inlineStr"/>
+      <c r="V50" t="inlineStr"/>
+      <c r="W50" t="inlineStr"/>
+      <c r="X50" t="inlineStr"/>
+      <c r="Y50" t="inlineStr"/>
+      <c r="Z50" t="inlineStr"/>
+      <c r="AA50" t="inlineStr"/>
+      <c r="AB50" t="inlineStr"/>
+      <c r="AC50" t="inlineStr"/>
+      <c r="AD50" t="inlineStr"/>
+      <c r="AE50" t="inlineStr"/>
+      <c r="AF50" t="inlineStr"/>
+      <c r="AG50" t="inlineStr"/>
+      <c r="AH50" t="inlineStr"/>
+      <c r="AI50" t="inlineStr"/>
+      <c r="AJ50" t="inlineStr"/>
+      <c r="AK50" t="inlineStr"/>
+      <c r="AL50" t="inlineStr"/>
+      <c r="AM50" t="inlineStr"/>
+      <c r="AN50" t="inlineStr"/>
+      <c r="AO50" t="inlineStr"/>
+      <c r="AP50" t="inlineStr"/>
+      <c r="AQ50" t="inlineStr"/>
+      <c r="AR50" t="inlineStr"/>
+      <c r="AS50" t="inlineStr"/>
+      <c r="AT50" t="inlineStr"/>
+      <c r="AU50" t="inlineStr"/>
+      <c r="AV50" t="inlineStr"/>
+      <c r="AW50" t="inlineStr"/>
+      <c r="AX50" t="inlineStr"/>
+      <c r="AY50" t="inlineStr"/>
+      <c r="AZ50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -6669,6 +7687,56 @@
           <t>Fast Break Points: Points scored by a player on a fast break. Includes points from FTs after a foul.</t>
         </is>
       </c>
+      <c r="C51" t="inlineStr"/>
+      <c r="D51" t="inlineStr"/>
+      <c r="E51" t="inlineStr"/>
+      <c r="F51" t="inlineStr"/>
+      <c r="G51" t="inlineStr"/>
+      <c r="H51" t="inlineStr"/>
+      <c r="I51" t="inlineStr"/>
+      <c r="J51" t="inlineStr"/>
+      <c r="K51" t="inlineStr"/>
+      <c r="L51" t="inlineStr"/>
+      <c r="M51" t="inlineStr"/>
+      <c r="N51" t="inlineStr"/>
+      <c r="O51" t="inlineStr"/>
+      <c r="P51" t="inlineStr"/>
+      <c r="Q51" t="inlineStr"/>
+      <c r="R51" t="inlineStr"/>
+      <c r="S51" t="inlineStr"/>
+      <c r="T51" t="inlineStr"/>
+      <c r="U51" t="inlineStr"/>
+      <c r="V51" t="inlineStr"/>
+      <c r="W51" t="inlineStr"/>
+      <c r="X51" t="inlineStr"/>
+      <c r="Y51" t="inlineStr"/>
+      <c r="Z51" t="inlineStr"/>
+      <c r="AA51" t="inlineStr"/>
+      <c r="AB51" t="inlineStr"/>
+      <c r="AC51" t="inlineStr"/>
+      <c r="AD51" t="inlineStr"/>
+      <c r="AE51" t="inlineStr"/>
+      <c r="AF51" t="inlineStr"/>
+      <c r="AG51" t="inlineStr"/>
+      <c r="AH51" t="inlineStr"/>
+      <c r="AI51" t="inlineStr"/>
+      <c r="AJ51" t="inlineStr"/>
+      <c r="AK51" t="inlineStr"/>
+      <c r="AL51" t="inlineStr"/>
+      <c r="AM51" t="inlineStr"/>
+      <c r="AN51" t="inlineStr"/>
+      <c r="AO51" t="inlineStr"/>
+      <c r="AP51" t="inlineStr"/>
+      <c r="AQ51" t="inlineStr"/>
+      <c r="AR51" t="inlineStr"/>
+      <c r="AS51" t="inlineStr"/>
+      <c r="AT51" t="inlineStr"/>
+      <c r="AU51" t="inlineStr"/>
+      <c r="AV51" t="inlineStr"/>
+      <c r="AW51" t="inlineStr"/>
+      <c r="AX51" t="inlineStr"/>
+      <c r="AY51" t="inlineStr"/>
+      <c r="AZ51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -6681,6 +7749,56 @@
           <t>Fast Break Opportunity: When a player scores a FG or is fouled on a fast break. A fast break is a play within 8 seconds of a DRB, STL, or opponent's made basket. 'And-one' plays are excluded.</t>
         </is>
       </c>
+      <c r="C52" t="inlineStr"/>
+      <c r="D52" t="inlineStr"/>
+      <c r="E52" t="inlineStr"/>
+      <c r="F52" t="inlineStr"/>
+      <c r="G52" t="inlineStr"/>
+      <c r="H52" t="inlineStr"/>
+      <c r="I52" t="inlineStr"/>
+      <c r="J52" t="inlineStr"/>
+      <c r="K52" t="inlineStr"/>
+      <c r="L52" t="inlineStr"/>
+      <c r="M52" t="inlineStr"/>
+      <c r="N52" t="inlineStr"/>
+      <c r="O52" t="inlineStr"/>
+      <c r="P52" t="inlineStr"/>
+      <c r="Q52" t="inlineStr"/>
+      <c r="R52" t="inlineStr"/>
+      <c r="S52" t="inlineStr"/>
+      <c r="T52" t="inlineStr"/>
+      <c r="U52" t="inlineStr"/>
+      <c r="V52" t="inlineStr"/>
+      <c r="W52" t="inlineStr"/>
+      <c r="X52" t="inlineStr"/>
+      <c r="Y52" t="inlineStr"/>
+      <c r="Z52" t="inlineStr"/>
+      <c r="AA52" t="inlineStr"/>
+      <c r="AB52" t="inlineStr"/>
+      <c r="AC52" t="inlineStr"/>
+      <c r="AD52" t="inlineStr"/>
+      <c r="AE52" t="inlineStr"/>
+      <c r="AF52" t="inlineStr"/>
+      <c r="AG52" t="inlineStr"/>
+      <c r="AH52" t="inlineStr"/>
+      <c r="AI52" t="inlineStr"/>
+      <c r="AJ52" t="inlineStr"/>
+      <c r="AK52" t="inlineStr"/>
+      <c r="AL52" t="inlineStr"/>
+      <c r="AM52" t="inlineStr"/>
+      <c r="AN52" t="inlineStr"/>
+      <c r="AO52" t="inlineStr"/>
+      <c r="AP52" t="inlineStr"/>
+      <c r="AQ52" t="inlineStr"/>
+      <c r="AR52" t="inlineStr"/>
+      <c r="AS52" t="inlineStr"/>
+      <c r="AT52" t="inlineStr"/>
+      <c r="AU52" t="inlineStr"/>
+      <c r="AV52" t="inlineStr"/>
+      <c r="AW52" t="inlineStr"/>
+      <c r="AX52" t="inlineStr"/>
+      <c r="AY52" t="inlineStr"/>
+      <c r="AZ52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -6693,6 +7811,56 @@
           <t>An estimate of possessions used by a player. Formula: FGA + (0.44 * FTA) + TO</t>
         </is>
       </c>
+      <c r="C53" t="inlineStr"/>
+      <c r="D53" t="inlineStr"/>
+      <c r="E53" t="inlineStr"/>
+      <c r="F53" t="inlineStr"/>
+      <c r="G53" t="inlineStr"/>
+      <c r="H53" t="inlineStr"/>
+      <c r="I53" t="inlineStr"/>
+      <c r="J53" t="inlineStr"/>
+      <c r="K53" t="inlineStr"/>
+      <c r="L53" t="inlineStr"/>
+      <c r="M53" t="inlineStr"/>
+      <c r="N53" t="inlineStr"/>
+      <c r="O53" t="inlineStr"/>
+      <c r="P53" t="inlineStr"/>
+      <c r="Q53" t="inlineStr"/>
+      <c r="R53" t="inlineStr"/>
+      <c r="S53" t="inlineStr"/>
+      <c r="T53" t="inlineStr"/>
+      <c r="U53" t="inlineStr"/>
+      <c r="V53" t="inlineStr"/>
+      <c r="W53" t="inlineStr"/>
+      <c r="X53" t="inlineStr"/>
+      <c r="Y53" t="inlineStr"/>
+      <c r="Z53" t="inlineStr"/>
+      <c r="AA53" t="inlineStr"/>
+      <c r="AB53" t="inlineStr"/>
+      <c r="AC53" t="inlineStr"/>
+      <c r="AD53" t="inlineStr"/>
+      <c r="AE53" t="inlineStr"/>
+      <c r="AF53" t="inlineStr"/>
+      <c r="AG53" t="inlineStr"/>
+      <c r="AH53" t="inlineStr"/>
+      <c r="AI53" t="inlineStr"/>
+      <c r="AJ53" t="inlineStr"/>
+      <c r="AK53" t="inlineStr"/>
+      <c r="AL53" t="inlineStr"/>
+      <c r="AM53" t="inlineStr"/>
+      <c r="AN53" t="inlineStr"/>
+      <c r="AO53" t="inlineStr"/>
+      <c r="AP53" t="inlineStr"/>
+      <c r="AQ53" t="inlineStr"/>
+      <c r="AR53" t="inlineStr"/>
+      <c r="AS53" t="inlineStr"/>
+      <c r="AT53" t="inlineStr"/>
+      <c r="AU53" t="inlineStr"/>
+      <c r="AV53" t="inlineStr"/>
+      <c r="AW53" t="inlineStr"/>
+      <c r="AX53" t="inlineStr"/>
+      <c r="AY53" t="inlineStr"/>
+      <c r="AZ53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -6705,6 +7873,56 @@
           <t>Effective Field Goal Percentage. Adjusts for the fact that a 3-point field goal is worth more than a 2-point field goal.</t>
         </is>
       </c>
+      <c r="C54" t="inlineStr"/>
+      <c r="D54" t="inlineStr"/>
+      <c r="E54" t="inlineStr"/>
+      <c r="F54" t="inlineStr"/>
+      <c r="G54" t="inlineStr"/>
+      <c r="H54" t="inlineStr"/>
+      <c r="I54" t="inlineStr"/>
+      <c r="J54" t="inlineStr"/>
+      <c r="K54" t="inlineStr"/>
+      <c r="L54" t="inlineStr"/>
+      <c r="M54" t="inlineStr"/>
+      <c r="N54" t="inlineStr"/>
+      <c r="O54" t="inlineStr"/>
+      <c r="P54" t="inlineStr"/>
+      <c r="Q54" t="inlineStr"/>
+      <c r="R54" t="inlineStr"/>
+      <c r="S54" t="inlineStr"/>
+      <c r="T54" t="inlineStr"/>
+      <c r="U54" t="inlineStr"/>
+      <c r="V54" t="inlineStr"/>
+      <c r="W54" t="inlineStr"/>
+      <c r="X54" t="inlineStr"/>
+      <c r="Y54" t="inlineStr"/>
+      <c r="Z54" t="inlineStr"/>
+      <c r="AA54" t="inlineStr"/>
+      <c r="AB54" t="inlineStr"/>
+      <c r="AC54" t="inlineStr"/>
+      <c r="AD54" t="inlineStr"/>
+      <c r="AE54" t="inlineStr"/>
+      <c r="AF54" t="inlineStr"/>
+      <c r="AG54" t="inlineStr"/>
+      <c r="AH54" t="inlineStr"/>
+      <c r="AI54" t="inlineStr"/>
+      <c r="AJ54" t="inlineStr"/>
+      <c r="AK54" t="inlineStr"/>
+      <c r="AL54" t="inlineStr"/>
+      <c r="AM54" t="inlineStr"/>
+      <c r="AN54" t="inlineStr"/>
+      <c r="AO54" t="inlineStr"/>
+      <c r="AP54" t="inlineStr"/>
+      <c r="AQ54" t="inlineStr"/>
+      <c r="AR54" t="inlineStr"/>
+      <c r="AS54" t="inlineStr"/>
+      <c r="AT54" t="inlineStr"/>
+      <c r="AU54" t="inlineStr"/>
+      <c r="AV54" t="inlineStr"/>
+      <c r="AW54" t="inlineStr"/>
+      <c r="AX54" t="inlineStr"/>
+      <c r="AY54" t="inlineStr"/>
+      <c r="AZ54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -6717,6 +7935,56 @@
           <t>True Shooting Percentage. Measures shooting efficiency, taking into account 2-pt, 3-pt, and free throws.</t>
         </is>
       </c>
+      <c r="C55" t="inlineStr"/>
+      <c r="D55" t="inlineStr"/>
+      <c r="E55" t="inlineStr"/>
+      <c r="F55" t="inlineStr"/>
+      <c r="G55" t="inlineStr"/>
+      <c r="H55" t="inlineStr"/>
+      <c r="I55" t="inlineStr"/>
+      <c r="J55" t="inlineStr"/>
+      <c r="K55" t="inlineStr"/>
+      <c r="L55" t="inlineStr"/>
+      <c r="M55" t="inlineStr"/>
+      <c r="N55" t="inlineStr"/>
+      <c r="O55" t="inlineStr"/>
+      <c r="P55" t="inlineStr"/>
+      <c r="Q55" t="inlineStr"/>
+      <c r="R55" t="inlineStr"/>
+      <c r="S55" t="inlineStr"/>
+      <c r="T55" t="inlineStr"/>
+      <c r="U55" t="inlineStr"/>
+      <c r="V55" t="inlineStr"/>
+      <c r="W55" t="inlineStr"/>
+      <c r="X55" t="inlineStr"/>
+      <c r="Y55" t="inlineStr"/>
+      <c r="Z55" t="inlineStr"/>
+      <c r="AA55" t="inlineStr"/>
+      <c r="AB55" t="inlineStr"/>
+      <c r="AC55" t="inlineStr"/>
+      <c r="AD55" t="inlineStr"/>
+      <c r="AE55" t="inlineStr"/>
+      <c r="AF55" t="inlineStr"/>
+      <c r="AG55" t="inlineStr"/>
+      <c r="AH55" t="inlineStr"/>
+      <c r="AI55" t="inlineStr"/>
+      <c r="AJ55" t="inlineStr"/>
+      <c r="AK55" t="inlineStr"/>
+      <c r="AL55" t="inlineStr"/>
+      <c r="AM55" t="inlineStr"/>
+      <c r="AN55" t="inlineStr"/>
+      <c r="AO55" t="inlineStr"/>
+      <c r="AP55" t="inlineStr"/>
+      <c r="AQ55" t="inlineStr"/>
+      <c r="AR55" t="inlineStr"/>
+      <c r="AS55" t="inlineStr"/>
+      <c r="AT55" t="inlineStr"/>
+      <c r="AU55" t="inlineStr"/>
+      <c r="AV55" t="inlineStr"/>
+      <c r="AW55" t="inlineStr"/>
+      <c r="AX55" t="inlineStr"/>
+      <c r="AY55" t="inlineStr"/>
+      <c r="AZ55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -6729,6 +7997,56 @@
           <t>Turnover Percentage. An estimate of turnovers per 100 plays.</t>
         </is>
       </c>
+      <c r="C56" t="inlineStr"/>
+      <c r="D56" t="inlineStr"/>
+      <c r="E56" t="inlineStr"/>
+      <c r="F56" t="inlineStr"/>
+      <c r="G56" t="inlineStr"/>
+      <c r="H56" t="inlineStr"/>
+      <c r="I56" t="inlineStr"/>
+      <c r="J56" t="inlineStr"/>
+      <c r="K56" t="inlineStr"/>
+      <c r="L56" t="inlineStr"/>
+      <c r="M56" t="inlineStr"/>
+      <c r="N56" t="inlineStr"/>
+      <c r="O56" t="inlineStr"/>
+      <c r="P56" t="inlineStr"/>
+      <c r="Q56" t="inlineStr"/>
+      <c r="R56" t="inlineStr"/>
+      <c r="S56" t="inlineStr"/>
+      <c r="T56" t="inlineStr"/>
+      <c r="U56" t="inlineStr"/>
+      <c r="V56" t="inlineStr"/>
+      <c r="W56" t="inlineStr"/>
+      <c r="X56" t="inlineStr"/>
+      <c r="Y56" t="inlineStr"/>
+      <c r="Z56" t="inlineStr"/>
+      <c r="AA56" t="inlineStr"/>
+      <c r="AB56" t="inlineStr"/>
+      <c r="AC56" t="inlineStr"/>
+      <c r="AD56" t="inlineStr"/>
+      <c r="AE56" t="inlineStr"/>
+      <c r="AF56" t="inlineStr"/>
+      <c r="AG56" t="inlineStr"/>
+      <c r="AH56" t="inlineStr"/>
+      <c r="AI56" t="inlineStr"/>
+      <c r="AJ56" t="inlineStr"/>
+      <c r="AK56" t="inlineStr"/>
+      <c r="AL56" t="inlineStr"/>
+      <c r="AM56" t="inlineStr"/>
+      <c r="AN56" t="inlineStr"/>
+      <c r="AO56" t="inlineStr"/>
+      <c r="AP56" t="inlineStr"/>
+      <c r="AQ56" t="inlineStr"/>
+      <c r="AR56" t="inlineStr"/>
+      <c r="AS56" t="inlineStr"/>
+      <c r="AT56" t="inlineStr"/>
+      <c r="AU56" t="inlineStr"/>
+      <c r="AV56" t="inlineStr"/>
+      <c r="AW56" t="inlineStr"/>
+      <c r="AX56" t="inlineStr"/>
+      <c r="AY56" t="inlineStr"/>
+      <c r="AZ56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -6741,6 +8059,56 @@
           <t>Free Throw Rate. How frequently a player scores from the free throw line relative to their field goal attempts.</t>
         </is>
       </c>
+      <c r="C57" t="inlineStr"/>
+      <c r="D57" t="inlineStr"/>
+      <c r="E57" t="inlineStr"/>
+      <c r="F57" t="inlineStr"/>
+      <c r="G57" t="inlineStr"/>
+      <c r="H57" t="inlineStr"/>
+      <c r="I57" t="inlineStr"/>
+      <c r="J57" t="inlineStr"/>
+      <c r="K57" t="inlineStr"/>
+      <c r="L57" t="inlineStr"/>
+      <c r="M57" t="inlineStr"/>
+      <c r="N57" t="inlineStr"/>
+      <c r="O57" t="inlineStr"/>
+      <c r="P57" t="inlineStr"/>
+      <c r="Q57" t="inlineStr"/>
+      <c r="R57" t="inlineStr"/>
+      <c r="S57" t="inlineStr"/>
+      <c r="T57" t="inlineStr"/>
+      <c r="U57" t="inlineStr"/>
+      <c r="V57" t="inlineStr"/>
+      <c r="W57" t="inlineStr"/>
+      <c r="X57" t="inlineStr"/>
+      <c r="Y57" t="inlineStr"/>
+      <c r="Z57" t="inlineStr"/>
+      <c r="AA57" t="inlineStr"/>
+      <c r="AB57" t="inlineStr"/>
+      <c r="AC57" t="inlineStr"/>
+      <c r="AD57" t="inlineStr"/>
+      <c r="AE57" t="inlineStr"/>
+      <c r="AF57" t="inlineStr"/>
+      <c r="AG57" t="inlineStr"/>
+      <c r="AH57" t="inlineStr"/>
+      <c r="AI57" t="inlineStr"/>
+      <c r="AJ57" t="inlineStr"/>
+      <c r="AK57" t="inlineStr"/>
+      <c r="AL57" t="inlineStr"/>
+      <c r="AM57" t="inlineStr"/>
+      <c r="AN57" t="inlineStr"/>
+      <c r="AO57" t="inlineStr"/>
+      <c r="AP57" t="inlineStr"/>
+      <c r="AQ57" t="inlineStr"/>
+      <c r="AR57" t="inlineStr"/>
+      <c r="AS57" t="inlineStr"/>
+      <c r="AT57" t="inlineStr"/>
+      <c r="AU57" t="inlineStr"/>
+      <c r="AV57" t="inlineStr"/>
+      <c r="AW57" t="inlineStr"/>
+      <c r="AX57" t="inlineStr"/>
+      <c r="AY57" t="inlineStr"/>
+      <c r="AZ57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -6753,6 +8121,56 @@
           <t>Assist to Turnover Ratio. A measure of a player's ball security and playmaking.</t>
         </is>
       </c>
+      <c r="C58" t="inlineStr"/>
+      <c r="D58" t="inlineStr"/>
+      <c r="E58" t="inlineStr"/>
+      <c r="F58" t="inlineStr"/>
+      <c r="G58" t="inlineStr"/>
+      <c r="H58" t="inlineStr"/>
+      <c r="I58" t="inlineStr"/>
+      <c r="J58" t="inlineStr"/>
+      <c r="K58" t="inlineStr"/>
+      <c r="L58" t="inlineStr"/>
+      <c r="M58" t="inlineStr"/>
+      <c r="N58" t="inlineStr"/>
+      <c r="O58" t="inlineStr"/>
+      <c r="P58" t="inlineStr"/>
+      <c r="Q58" t="inlineStr"/>
+      <c r="R58" t="inlineStr"/>
+      <c r="S58" t="inlineStr"/>
+      <c r="T58" t="inlineStr"/>
+      <c r="U58" t="inlineStr"/>
+      <c r="V58" t="inlineStr"/>
+      <c r="W58" t="inlineStr"/>
+      <c r="X58" t="inlineStr"/>
+      <c r="Y58" t="inlineStr"/>
+      <c r="Z58" t="inlineStr"/>
+      <c r="AA58" t="inlineStr"/>
+      <c r="AB58" t="inlineStr"/>
+      <c r="AC58" t="inlineStr"/>
+      <c r="AD58" t="inlineStr"/>
+      <c r="AE58" t="inlineStr"/>
+      <c r="AF58" t="inlineStr"/>
+      <c r="AG58" t="inlineStr"/>
+      <c r="AH58" t="inlineStr"/>
+      <c r="AI58" t="inlineStr"/>
+      <c r="AJ58" t="inlineStr"/>
+      <c r="AK58" t="inlineStr"/>
+      <c r="AL58" t="inlineStr"/>
+      <c r="AM58" t="inlineStr"/>
+      <c r="AN58" t="inlineStr"/>
+      <c r="AO58" t="inlineStr"/>
+      <c r="AP58" t="inlineStr"/>
+      <c r="AQ58" t="inlineStr"/>
+      <c r="AR58" t="inlineStr"/>
+      <c r="AS58" t="inlineStr"/>
+      <c r="AT58" t="inlineStr"/>
+      <c r="AU58" t="inlineStr"/>
+      <c r="AV58" t="inlineStr"/>
+      <c r="AW58" t="inlineStr"/>
+      <c r="AX58" t="inlineStr"/>
+      <c r="AY58" t="inlineStr"/>
+      <c r="AZ58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -6765,6 +8183,56 @@
           <t>Shot to Turnover Ratio. The number of field goal attempts a player takes for every turnover they commit.</t>
         </is>
       </c>
+      <c r="C59" t="inlineStr"/>
+      <c r="D59" t="inlineStr"/>
+      <c r="E59" t="inlineStr"/>
+      <c r="F59" t="inlineStr"/>
+      <c r="G59" t="inlineStr"/>
+      <c r="H59" t="inlineStr"/>
+      <c r="I59" t="inlineStr"/>
+      <c r="J59" t="inlineStr"/>
+      <c r="K59" t="inlineStr"/>
+      <c r="L59" t="inlineStr"/>
+      <c r="M59" t="inlineStr"/>
+      <c r="N59" t="inlineStr"/>
+      <c r="O59" t="inlineStr"/>
+      <c r="P59" t="inlineStr"/>
+      <c r="Q59" t="inlineStr"/>
+      <c r="R59" t="inlineStr"/>
+      <c r="S59" t="inlineStr"/>
+      <c r="T59" t="inlineStr"/>
+      <c r="U59" t="inlineStr"/>
+      <c r="V59" t="inlineStr"/>
+      <c r="W59" t="inlineStr"/>
+      <c r="X59" t="inlineStr"/>
+      <c r="Y59" t="inlineStr"/>
+      <c r="Z59" t="inlineStr"/>
+      <c r="AA59" t="inlineStr"/>
+      <c r="AB59" t="inlineStr"/>
+      <c r="AC59" t="inlineStr"/>
+      <c r="AD59" t="inlineStr"/>
+      <c r="AE59" t="inlineStr"/>
+      <c r="AF59" t="inlineStr"/>
+      <c r="AG59" t="inlineStr"/>
+      <c r="AH59" t="inlineStr"/>
+      <c r="AI59" t="inlineStr"/>
+      <c r="AJ59" t="inlineStr"/>
+      <c r="AK59" t="inlineStr"/>
+      <c r="AL59" t="inlineStr"/>
+      <c r="AM59" t="inlineStr"/>
+      <c r="AN59" t="inlineStr"/>
+      <c r="AO59" t="inlineStr"/>
+      <c r="AP59" t="inlineStr"/>
+      <c r="AQ59" t="inlineStr"/>
+      <c r="AR59" t="inlineStr"/>
+      <c r="AS59" t="inlineStr"/>
+      <c r="AT59" t="inlineStr"/>
+      <c r="AU59" t="inlineStr"/>
+      <c r="AV59" t="inlineStr"/>
+      <c r="AW59" t="inlineStr"/>
+      <c r="AX59" t="inlineStr"/>
+      <c r="AY59" t="inlineStr"/>
+      <c r="AZ59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -6777,6 +8245,56 @@
           <t>Generated Offense to Turnover Ratio. The number of shots and assists a player generates for every turnover.</t>
         </is>
       </c>
+      <c r="C60" t="inlineStr"/>
+      <c r="D60" t="inlineStr"/>
+      <c r="E60" t="inlineStr"/>
+      <c r="F60" t="inlineStr"/>
+      <c r="G60" t="inlineStr"/>
+      <c r="H60" t="inlineStr"/>
+      <c r="I60" t="inlineStr"/>
+      <c r="J60" t="inlineStr"/>
+      <c r="K60" t="inlineStr"/>
+      <c r="L60" t="inlineStr"/>
+      <c r="M60" t="inlineStr"/>
+      <c r="N60" t="inlineStr"/>
+      <c r="O60" t="inlineStr"/>
+      <c r="P60" t="inlineStr"/>
+      <c r="Q60" t="inlineStr"/>
+      <c r="R60" t="inlineStr"/>
+      <c r="S60" t="inlineStr"/>
+      <c r="T60" t="inlineStr"/>
+      <c r="U60" t="inlineStr"/>
+      <c r="V60" t="inlineStr"/>
+      <c r="W60" t="inlineStr"/>
+      <c r="X60" t="inlineStr"/>
+      <c r="Y60" t="inlineStr"/>
+      <c r="Z60" t="inlineStr"/>
+      <c r="AA60" t="inlineStr"/>
+      <c r="AB60" t="inlineStr"/>
+      <c r="AC60" t="inlineStr"/>
+      <c r="AD60" t="inlineStr"/>
+      <c r="AE60" t="inlineStr"/>
+      <c r="AF60" t="inlineStr"/>
+      <c r="AG60" t="inlineStr"/>
+      <c r="AH60" t="inlineStr"/>
+      <c r="AI60" t="inlineStr"/>
+      <c r="AJ60" t="inlineStr"/>
+      <c r="AK60" t="inlineStr"/>
+      <c r="AL60" t="inlineStr"/>
+      <c r="AM60" t="inlineStr"/>
+      <c r="AN60" t="inlineStr"/>
+      <c r="AO60" t="inlineStr"/>
+      <c r="AP60" t="inlineStr"/>
+      <c r="AQ60" t="inlineStr"/>
+      <c r="AR60" t="inlineStr"/>
+      <c r="AS60" t="inlineStr"/>
+      <c r="AT60" t="inlineStr"/>
+      <c r="AU60" t="inlineStr"/>
+      <c r="AV60" t="inlineStr"/>
+      <c r="AW60" t="inlineStr"/>
+      <c r="AX60" t="inlineStr"/>
+      <c r="AY60" t="inlineStr"/>
+      <c r="AZ60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -6789,6 +8307,56 @@
           <t>Usage Rate. An estimate of the percentage of a team's offensive possessions a player 'uses' while on the floor.</t>
         </is>
       </c>
+      <c r="C61" t="inlineStr"/>
+      <c r="D61" t="inlineStr"/>
+      <c r="E61" t="inlineStr"/>
+      <c r="F61" t="inlineStr"/>
+      <c r="G61" t="inlineStr"/>
+      <c r="H61" t="inlineStr"/>
+      <c r="I61" t="inlineStr"/>
+      <c r="J61" t="inlineStr"/>
+      <c r="K61" t="inlineStr"/>
+      <c r="L61" t="inlineStr"/>
+      <c r="M61" t="inlineStr"/>
+      <c r="N61" t="inlineStr"/>
+      <c r="O61" t="inlineStr"/>
+      <c r="P61" t="inlineStr"/>
+      <c r="Q61" t="inlineStr"/>
+      <c r="R61" t="inlineStr"/>
+      <c r="S61" t="inlineStr"/>
+      <c r="T61" t="inlineStr"/>
+      <c r="U61" t="inlineStr"/>
+      <c r="V61" t="inlineStr"/>
+      <c r="W61" t="inlineStr"/>
+      <c r="X61" t="inlineStr"/>
+      <c r="Y61" t="inlineStr"/>
+      <c r="Z61" t="inlineStr"/>
+      <c r="AA61" t="inlineStr"/>
+      <c r="AB61" t="inlineStr"/>
+      <c r="AC61" t="inlineStr"/>
+      <c r="AD61" t="inlineStr"/>
+      <c r="AE61" t="inlineStr"/>
+      <c r="AF61" t="inlineStr"/>
+      <c r="AG61" t="inlineStr"/>
+      <c r="AH61" t="inlineStr"/>
+      <c r="AI61" t="inlineStr"/>
+      <c r="AJ61" t="inlineStr"/>
+      <c r="AK61" t="inlineStr"/>
+      <c r="AL61" t="inlineStr"/>
+      <c r="AM61" t="inlineStr"/>
+      <c r="AN61" t="inlineStr"/>
+      <c r="AO61" t="inlineStr"/>
+      <c r="AP61" t="inlineStr"/>
+      <c r="AQ61" t="inlineStr"/>
+      <c r="AR61" t="inlineStr"/>
+      <c r="AS61" t="inlineStr"/>
+      <c r="AT61" t="inlineStr"/>
+      <c r="AU61" t="inlineStr"/>
+      <c r="AV61" t="inlineStr"/>
+      <c r="AW61" t="inlineStr"/>
+      <c r="AX61" t="inlineStr"/>
+      <c r="AY61" t="inlineStr"/>
+      <c r="AZ61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -6801,6 +8369,56 @@
           <t>Offensive/Defensive Rebound Percentage. Percentage of available offensive/defensive rebounds a player secured while on the floor.</t>
         </is>
       </c>
+      <c r="C62" t="inlineStr"/>
+      <c r="D62" t="inlineStr"/>
+      <c r="E62" t="inlineStr"/>
+      <c r="F62" t="inlineStr"/>
+      <c r="G62" t="inlineStr"/>
+      <c r="H62" t="inlineStr"/>
+      <c r="I62" t="inlineStr"/>
+      <c r="J62" t="inlineStr"/>
+      <c r="K62" t="inlineStr"/>
+      <c r="L62" t="inlineStr"/>
+      <c r="M62" t="inlineStr"/>
+      <c r="N62" t="inlineStr"/>
+      <c r="O62" t="inlineStr"/>
+      <c r="P62" t="inlineStr"/>
+      <c r="Q62" t="inlineStr"/>
+      <c r="R62" t="inlineStr"/>
+      <c r="S62" t="inlineStr"/>
+      <c r="T62" t="inlineStr"/>
+      <c r="U62" t="inlineStr"/>
+      <c r="V62" t="inlineStr"/>
+      <c r="W62" t="inlineStr"/>
+      <c r="X62" t="inlineStr"/>
+      <c r="Y62" t="inlineStr"/>
+      <c r="Z62" t="inlineStr"/>
+      <c r="AA62" t="inlineStr"/>
+      <c r="AB62" t="inlineStr"/>
+      <c r="AC62" t="inlineStr"/>
+      <c r="AD62" t="inlineStr"/>
+      <c r="AE62" t="inlineStr"/>
+      <c r="AF62" t="inlineStr"/>
+      <c r="AG62" t="inlineStr"/>
+      <c r="AH62" t="inlineStr"/>
+      <c r="AI62" t="inlineStr"/>
+      <c r="AJ62" t="inlineStr"/>
+      <c r="AK62" t="inlineStr"/>
+      <c r="AL62" t="inlineStr"/>
+      <c r="AM62" t="inlineStr"/>
+      <c r="AN62" t="inlineStr"/>
+      <c r="AO62" t="inlineStr"/>
+      <c r="AP62" t="inlineStr"/>
+      <c r="AQ62" t="inlineStr"/>
+      <c r="AR62" t="inlineStr"/>
+      <c r="AS62" t="inlineStr"/>
+      <c r="AT62" t="inlineStr"/>
+      <c r="AU62" t="inlineStr"/>
+      <c r="AV62" t="inlineStr"/>
+      <c r="AW62" t="inlineStr"/>
+      <c r="AX62" t="inlineStr"/>
+      <c r="AY62" t="inlineStr"/>
+      <c r="AZ62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -6813,6 +8431,56 @@
           <t>Assist Percentage. An estimate of the percentage of teammate field goals a player assisted on while on the floor.</t>
         </is>
       </c>
+      <c r="C63" t="inlineStr"/>
+      <c r="D63" t="inlineStr"/>
+      <c r="E63" t="inlineStr"/>
+      <c r="F63" t="inlineStr"/>
+      <c r="G63" t="inlineStr"/>
+      <c r="H63" t="inlineStr"/>
+      <c r="I63" t="inlineStr"/>
+      <c r="J63" t="inlineStr"/>
+      <c r="K63" t="inlineStr"/>
+      <c r="L63" t="inlineStr"/>
+      <c r="M63" t="inlineStr"/>
+      <c r="N63" t="inlineStr"/>
+      <c r="O63" t="inlineStr"/>
+      <c r="P63" t="inlineStr"/>
+      <c r="Q63" t="inlineStr"/>
+      <c r="R63" t="inlineStr"/>
+      <c r="S63" t="inlineStr"/>
+      <c r="T63" t="inlineStr"/>
+      <c r="U63" t="inlineStr"/>
+      <c r="V63" t="inlineStr"/>
+      <c r="W63" t="inlineStr"/>
+      <c r="X63" t="inlineStr"/>
+      <c r="Y63" t="inlineStr"/>
+      <c r="Z63" t="inlineStr"/>
+      <c r="AA63" t="inlineStr"/>
+      <c r="AB63" t="inlineStr"/>
+      <c r="AC63" t="inlineStr"/>
+      <c r="AD63" t="inlineStr"/>
+      <c r="AE63" t="inlineStr"/>
+      <c r="AF63" t="inlineStr"/>
+      <c r="AG63" t="inlineStr"/>
+      <c r="AH63" t="inlineStr"/>
+      <c r="AI63" t="inlineStr"/>
+      <c r="AJ63" t="inlineStr"/>
+      <c r="AK63" t="inlineStr"/>
+      <c r="AL63" t="inlineStr"/>
+      <c r="AM63" t="inlineStr"/>
+      <c r="AN63" t="inlineStr"/>
+      <c r="AO63" t="inlineStr"/>
+      <c r="AP63" t="inlineStr"/>
+      <c r="AQ63" t="inlineStr"/>
+      <c r="AR63" t="inlineStr"/>
+      <c r="AS63" t="inlineStr"/>
+      <c r="AT63" t="inlineStr"/>
+      <c r="AU63" t="inlineStr"/>
+      <c r="AV63" t="inlineStr"/>
+      <c r="AW63" t="inlineStr"/>
+      <c r="AX63" t="inlineStr"/>
+      <c r="AY63" t="inlineStr"/>
+      <c r="AZ63" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>